<commit_message>
Publish updated LTI communication
</commit_message>
<xml_diff>
--- a/lti/downloads/Aivel_LTI_calculator_v2.xlsx
+++ b/lti/downloads/Aivel_LTI_calculator_v2.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Калькулятор" sheetId="1" r:id="R98914e4c08fd4f01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Один пакет" sheetId="2" r:id="R290643b75cd1420a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Правила и сверка" sheetId="3" r:id="Rf2195f6e32914d1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ежегодные циклы" sheetId="4" r:id="R9cc63188a5974d32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Резерв и пять лет" sheetId="5" r:id="Raf3c3d2e93d1424c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Калькулятор" sheetId="1" r:id="R3b5c16e8f75f44c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Один пакет" sheetId="2" r:id="R50f2bc9534c64cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Правила и сверка" sheetId="3" r:id="Rb8703d09b7cc4b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ежегодные циклы" sheetId="4" r:id="R9e706a2564154aed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Резерв и пять лет" sheetId="5" r:id="R6b8dc65f0d9b49c3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -462,7 +462,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="81">
+  <x:fills count="90">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -864,6 +864,51 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2F5597"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF5B9BD5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="14">
     <x:border/>
@@ -991,7 +1036,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="1142">
+  <x:cellXfs count="1339">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3674,6 +3719,511 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="210" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="36" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="83" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="84" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="4" fillId="84" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="4" fillId="84" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="84" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="4" fillId="84" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="4" fillId="84" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="85" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="37" fillId="82" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="37" fillId="82" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="38" fillId="82" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="37" fillId="82" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="37" fillId="82" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="85" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="22" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="42" fillId="84" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="42" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="39" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="39" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="39" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="39" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="42" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="42" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="42" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="40" fillId="82" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="47" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="47" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="47" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="47" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="84" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="40" fillId="84" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="40" fillId="84" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="40" fillId="84" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="10" fontId="6" fillId="84" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="41" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="210" fontId="41" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="41" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="3" fillId="81" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="1" fontId="39" fillId="81" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="39" fillId="81" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="39" fillId="81" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="3" fillId="81" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="3" fillId="81" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="47" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="62" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="62" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="47" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="208" fontId="5" fillId="85" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="47" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="48" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="49" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="20" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="14" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="20" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="84" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="43" fillId="84" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="43" fillId="84" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="212" fontId="43" fillId="84" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="47" fillId="84" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="43" fillId="84" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="43" fillId="84" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="43" fillId="84" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="84" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="47" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="28" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="31" fillId="85" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="53" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="33" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="54" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="34" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="34" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="56" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="56" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="34" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="34" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="59" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="56" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="56" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="59" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="59" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="56" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="34" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="60" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="56" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="56" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="60" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="60" fillId="81" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="89" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="35" fillId="89" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="89" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="89" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="32" fillId="89" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="85" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="30" fillId="85" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="43" fillId="84" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="51" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="51" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="51" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="59" fillId="87" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="207" fontId="23" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="23" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="23" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="87" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="23" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="211" fontId="23" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="23" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="86" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="47" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="47" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="47" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="47" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="47" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="47" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="47" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="47" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="49" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="46" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="47" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="47" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="47" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="47" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="48" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="48" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="48" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="48" fillId="86" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="61" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="47" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="47" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="47" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="47" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="61" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="61" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="61" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="61" fillId="88" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="49" fillId="87" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="89" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="89" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="89" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="5" fillId="85" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="22" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="22" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="62" fillId="82" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="47" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="47" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="5" fillId="85" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="5" fillId="85" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="47" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="47" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="47" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="47" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="47" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="47" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="43" fillId="84" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="57" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="211" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="210" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="209" fontId="5" fillId="83" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="6" fillId="89" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="89" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="89" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -4064,8 +4614,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
-      <x:c r="A1" s="898" t="str">
-        <x:v>LTI: пятилетняя ёмкость резерва — 15 участников ежегодно</x:v>
+      <x:c r="A1" s="1142" t="str">
+        <x:v>LTI: пятилетняя ёмкость резерва — 59 решений за пять лет</x:v>
       </x:c>
       <x:c r="B1" s="38"/>
       <x:c r="C1" s="38"/>
@@ -4080,68 +4630,68 @@
       <x:c r="L1" s="38"/>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
-      <x:c r="A2" s="899" t="str">
-        <x:v>Базовый сценарий: пять раундов, средний пакет 0,7 годового оклада, продажа сразу после пятого года. Голубые ячейки — пользовательские допущения.</x:v>
-      </x:c>
-      <x:c r="B2" s="899"/>
-      <x:c r="C2" s="899"/>
-      <x:c r="D2" s="899"/>
-      <x:c r="E2" s="899"/>
-      <x:c r="F2" s="899"/>
-      <x:c r="G2" s="899"/>
-      <x:c r="H2" s="899"/>
-      <x:c r="I2" s="899"/>
-      <x:c r="J2" s="899"/>
-      <x:c r="K2" s="899"/>
-      <x:c r="L2" s="899"/>
+      <x:c r="A2" s="1143" t="str">
+        <x:v>Базовый сценарий: 8 → 12 → 12 → 12 → 15 участников, максимальный целевой пакет 1,0 годового оклада, продажа сразу после пятого года. Голубые ячейки — пользовательские допущения.</x:v>
+      </x:c>
+      <x:c r="B2" s="1143"/>
+      <x:c r="C2" s="1143"/>
+      <x:c r="D2" s="1143"/>
+      <x:c r="E2" s="1143"/>
+      <x:c r="F2" s="1143"/>
+      <x:c r="G2" s="1143"/>
+      <x:c r="H2" s="1143"/>
+      <x:c r="I2" s="1143"/>
+      <x:c r="J2" s="1143"/>
+      <x:c r="K2" s="1143"/>
+      <x:c r="L2" s="1143"/>
     </x:row>
     <x:row r="4" ht="15" customHeight="1">
-      <x:c r="A4" s="900" t="str">
+      <x:c r="A4" s="1144" t="str">
         <x:v>Использовано резерва к концу 5-го года</x:v>
       </x:c>
-      <x:c r="B4" s="900"/>
-      <x:c r="C4" s="900"/>
-      <x:c r="D4" s="900" t="str">
+      <x:c r="B4" s="1144"/>
+      <x:c r="C4" s="1144"/>
+      <x:c r="D4" s="1144" t="str">
         <x:v>Свободный резерв, млн расчётных единиц</x:v>
       </x:c>
-      <x:c r="E4" s="900"/>
-      <x:c r="F4" s="900"/>
-      <x:c r="G4" s="900" t="str">
+      <x:c r="E4" s="1144"/>
+      <x:c r="F4" s="1144"/>
+      <x:c r="G4" s="1144" t="str">
         <x:v>Размытие исходной структуры</x:v>
       </x:c>
-      <x:c r="H4" s="900"/>
-      <x:c r="I4" s="900"/>
-      <x:c r="J4" s="900" t="str">
+      <x:c r="H4" s="1144"/>
+      <x:c r="I4" s="1144"/>
+      <x:c r="J4" s="1144" t="str">
         <x:v>Закрепившаяся стоимость при продаже, млн ₽</x:v>
       </x:c>
-      <x:c r="K4" s="900"/>
-      <x:c r="L4" s="900"/>
+      <x:c r="K4" s="1144"/>
+      <x:c r="L4" s="1144"/>
     </x:row>
     <x:row r="5" ht="15" customHeight="1">
-      <x:c r="A5" s="901" t="n">
+      <x:c r="A5" s="1145" t="n">
         <x:f>H27</x:f>
-        <x:v>0.9594484660512796</x:v>
-      </x:c>
-      <x:c r="B5" s="902"/>
-      <x:c r="C5" s="902"/>
-      <x:c r="D5" s="903" t="n">
+        <x:v>0.9504543051104589</x:v>
+      </x:c>
+      <x:c r="B5" s="1146"/>
+      <x:c r="C5" s="1146"/>
+      <x:c r="D5" s="1147" t="n">
         <x:f>I27</x:f>
-        <x:v>0.405515339487204</x:v>
-      </x:c>
-      <x:c r="E5" s="904"/>
-      <x:c r="F5" s="904"/>
-      <x:c r="G5" s="901" t="n">
+        <x:v>0.49545694889541103</x:v>
+      </x:c>
+      <x:c r="E5" s="1148"/>
+      <x:c r="F5" s="1148"/>
+      <x:c r="G5" s="1145" t="n">
         <x:f>L14</x:f>
         <x:v>0.5135685144200788</x:v>
       </x:c>
-      <x:c r="H5" s="901"/>
-      <x:c r="I5" s="901"/>
-      <x:c r="J5" s="905" t="n">
+      <x:c r="H5" s="1145"/>
+      <x:c r="I5" s="1145"/>
+      <x:c r="J5" s="1149" t="n">
         <x:f>L27</x:f>
-        <x:v>606.168263641155</x:v>
-      </x:c>
-      <x:c r="K5" s="906"/>
-      <x:c r="L5" s="906"/>
+        <x:v>563.0486670542933</x:v>
+      </x:c>
+      <x:c r="K5" s="1150"/>
+      <x:c r="L5" s="1150"/>
     </x:row>
     <x:row r="6" ht="15" customHeight="1">
       <x:c r="A6" s="34"/>
@@ -4158,54 +4708,54 @@
       <x:c r="L6" s="37"/>
     </x:row>
     <x:row r="8" ht="21.75" customHeight="1">
-      <x:c r="A8" s="907" t="str">
+      <x:c r="A8" s="1151" t="str">
         <x:v>1. Допущения и пять раундов финансирования</x:v>
       </x:c>
-      <x:c r="B8" s="907"/>
-      <x:c r="C8" s="907"/>
-      <x:c r="D8" s="907"/>
-      <x:c r="E8" s="907"/>
-      <x:c r="F8" s="907"/>
-      <x:c r="G8" s="907"/>
-      <x:c r="H8" s="907"/>
-      <x:c r="I8" s="907"/>
-      <x:c r="J8" s="907"/>
-      <x:c r="K8" s="907"/>
-      <x:c r="L8" s="907"/>
+      <x:c r="B8" s="1151"/>
+      <x:c r="C8" s="1151"/>
+      <x:c r="D8" s="1151"/>
+      <x:c r="E8" s="1151"/>
+      <x:c r="F8" s="1151"/>
+      <x:c r="G8" s="1151"/>
+      <x:c r="H8" s="1151"/>
+      <x:c r="I8" s="1151"/>
+      <x:c r="J8" s="1151"/>
+      <x:c r="K8" s="1151"/>
+      <x:c r="L8" s="1151"/>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
-      <x:c r="A9" s="908" t="str">
+      <x:c r="A9" s="1152" t="str">
         <x:v>Параметр</x:v>
       </x:c>
-      <x:c r="B9" s="908" t="str">
+      <x:c r="B9" s="1152" t="str">
         <x:v>Значение</x:v>
       </x:c>
       <x:c r="C9" s="2"/>
-      <x:c r="D9" s="908" t="str">
+      <x:c r="D9" s="1152" t="str">
         <x:v>Год</x:v>
       </x:c>
-      <x:c r="E9" s="914" t="str">
+      <x:c r="E9" s="1158" t="str">
         <x:v>Оценка до раунда, млн ₽</x:v>
       </x:c>
-      <x:c r="F9" s="908" t="str">
+      <x:c r="F9" s="1152" t="str">
         <x:v>Привлечено, млн ₽</x:v>
       </x:c>
-      <x:c r="G9" s="908" t="str">
+      <x:c r="G9" s="1152" t="str">
         <x:v>Оценка после раунда, млн ₽</x:v>
       </x:c>
-      <x:c r="H9" s="908" t="str">
+      <x:c r="H9" s="1152" t="str">
         <x:v>Расчётных единиц до раунда, млн</x:v>
       </x:c>
-      <x:c r="I9" s="908" t="str">
+      <x:c r="I9" s="1152" t="str">
         <x:v>Цена расчётной единицы, ₽</x:v>
       </x:c>
-      <x:c r="J9" s="908" t="str">
+      <x:c r="J9" s="1152" t="str">
         <x:v>Расчётных единиц инвестора, млн</x:v>
       </x:c>
-      <x:c r="K9" s="908" t="str">
+      <x:c r="K9" s="1152" t="str">
         <x:v>Расчётных единиц после раунда, млн</x:v>
       </x:c>
-      <x:c r="L9" s="908" t="str">
+      <x:c r="L9" s="1152" t="str">
         <x:v>Размытие исходной структуры</x:v>
       </x:c>
     </x:row>
@@ -4213,17 +4763,17 @@
       <x:c r="A10" s="3" t="str">
         <x:v>Расчётных единиц до 1-го раунда, млн</x:v>
       </x:c>
-      <x:c r="B10" s="909" t="n">
+      <x:c r="B10" s="1153" t="n">
         <x:v>100</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="5" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E10" s="915" t="n">
+      <x:c r="E10" s="1159" t="n">
         <x:v>1200</x:v>
       </x:c>
-      <x:c r="F10" s="909" t="n">
+      <x:c r="F10" s="1153" t="n">
         <x:v>400</x:v>
       </x:c>
       <x:c r="G10" s="242" t="n">
@@ -4255,17 +4805,17 @@
       <x:c r="A11" s="8" t="str">
         <x:v>Резерв LTI, млн расчётных единиц</x:v>
       </x:c>
-      <x:c r="B11" s="909" t="n">
+      <x:c r="B11" s="1153" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C11" s="8"/>
       <x:c r="D11" s="9" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E11" s="915" t="n">
+      <x:c r="E11" s="1159" t="n">
         <x:v>3200</x:v>
       </x:c>
-      <x:c r="F11" s="909" t="n">
+      <x:c r="F11" s="1153" t="n">
         <x:v>400</x:v>
       </x:c>
       <x:c r="G11" s="242" t="n">
@@ -4295,19 +4845,19 @@
     </x:row>
     <x:row r="12" ht="21.75" customHeight="1">
       <x:c r="A12" s="3" t="str">
-        <x:v>Участников ежегодно</x:v>
-      </x:c>
-      <x:c r="B12" s="910" t="n">
-        <x:v>15</x:v>
+        <x:v>Обычный предел участников за год</x:v>
+      </x:c>
+      <x:c r="B12" s="1154" t="n">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C12" s="3"/>
       <x:c r="D12" s="7" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E12" s="915" t="n">
+      <x:c r="E12" s="1159" t="n">
         <x:v>5760</x:v>
       </x:c>
-      <x:c r="F12" s="909" t="n">
+      <x:c r="F12" s="1153" t="n">
         <x:v>600</x:v>
       </x:c>
       <x:c r="G12" s="242" t="n">
@@ -4339,17 +4889,17 @@
       <x:c r="A13" s="8" t="str">
         <x:v>Годовой фиксированный оклад, млн ₽</x:v>
       </x:c>
-      <x:c r="B13" s="911" t="n">
+      <x:c r="B13" s="1155" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C13" s="8"/>
       <x:c r="D13" s="7" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E13" s="915" t="n">
+      <x:c r="E13" s="1159" t="n">
         <x:v>9216</x:v>
       </x:c>
-      <x:c r="F13" s="909" t="n">
+      <x:c r="F13" s="1153" t="n">
         <x:v>1000</x:v>
       </x:c>
       <x:c r="G13" s="268" t="n">
@@ -4379,19 +4929,19 @@
     </x:row>
     <x:row r="14" ht="14.399999618530273" hidden="0" customHeight="1">
       <x:c r="A14" s="3" t="str">
-        <x:v>Средний множитель пакета, ×</x:v>
-      </x:c>
-      <x:c r="B14" s="912" t="n">
-        <x:v>0.7</x:v>
+        <x:v>Максимальный целевой множитель пакета, ×</x:v>
+      </x:c>
+      <x:c r="B14" s="1156" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C14" s="89"/>
       <x:c r="D14" s="51" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E14" s="915" t="n">
+      <x:c r="E14" s="1159" t="n">
         <x:v>13363.2</x:v>
       </x:c>
-      <x:c r="F14" s="915" t="n">
+      <x:c r="F14" s="1159" t="n">
         <x:v>1600</x:v>
       </x:c>
       <x:c r="G14" s="243" t="n">
@@ -4421,100 +4971,100 @@
     </x:row>
     <x:row r="15" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A15" s="8" t="str">
-        <x:v>Средний пакет на человека, млн ₽</x:v>
+        <x:v>Максимальный целевой пакет на человека, млн ₽</x:v>
       </x:c>
       <x:c r="B15" s="241" t="n">
         <x:f>B13*B14</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C15" s="90"/>
-      <x:c r="D15" s="916" t="str">
+      <x:c r="D15" s="1160" t="str">
         <x:v>ИТОГО / ПРОДАЖА</x:v>
       </x:c>
-      <x:c r="E15" s="917"/>
-      <x:c r="F15" s="918" t="n">
+      <x:c r="E15" s="1161"/>
+      <x:c r="F15" s="1162" t="n">
         <x:f>SUM(F10:F14)</x:f>
         <x:v>4000</x:v>
       </x:c>
-      <x:c r="G15" s="918" t="n">
+      <x:c r="G15" s="1162" t="n">
         <x:f>G14</x:f>
         <x:v>14963.2</x:v>
       </x:c>
-      <x:c r="H15" s="918" t="n">
+      <x:c r="H15" s="1162" t="n">
         <x:f>H10</x:f>
         <x:v>100</x:v>
       </x:c>
-      <x:c r="I15" s="923" t="n">
+      <x:c r="I15" s="1167" t="n">
         <x:f>$B$19/K14</x:f>
         <x:v>77.8290376927874</x:v>
       </x:c>
-      <x:c r="J15" s="924" t="n">
+      <x:c r="J15" s="1168" t="n">
         <x:f>SUM(J10:J14)</x:f>
         <x:v>105.57879776384233</x:v>
       </x:c>
-      <x:c r="K15" s="924" t="n">
+      <x:c r="K15" s="1168" t="n">
         <x:f>K14</x:f>
         <x:v>205.57879776384232</x:v>
       </x:c>
-      <x:c r="L15" s="925" t="n">
+      <x:c r="L15" s="1169" t="n">
         <x:f>L14</x:f>
         <x:v>0.5135685144200788</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A16" s="3" t="str">
-        <x:v>Пакеты на год, млн ₽</x:v>
+        <x:v>Максимальный объём 59 решений, млн ₽</x:v>
       </x:c>
       <x:c r="B16" s="242" t="n">
-        <x:f>B12*B15</x:f>
-        <x:v>52.5</x:v>
+        <x:f>SUM(B22:B26)*B15</x:f>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="C16" s="89"/>
-      <x:c r="D16" s="1130"/>
-      <x:c r="E16" s="1131"/>
-      <x:c r="F16" s="1132"/>
-      <x:c r="G16" s="1132"/>
-      <x:c r="H16" s="1132"/>
-      <x:c r="I16" s="1132"/>
-      <x:c r="J16" s="1132"/>
-      <x:c r="K16" s="1132"/>
-      <x:c r="L16" s="1132"/>
+      <x:c r="D16" s="1333"/>
+      <x:c r="E16" s="1334"/>
+      <x:c r="F16" s="1335"/>
+      <x:c r="G16" s="1335"/>
+      <x:c r="H16" s="1335"/>
+      <x:c r="I16" s="1335"/>
+      <x:c r="J16" s="1335"/>
+      <x:c r="K16" s="1335"/>
+      <x:c r="L16" s="1335"/>
     </x:row>
     <x:row r="17" ht="40.5" hidden="0" customHeight="1">
       <x:c r="A17" s="90" t="str">
         <x:v>Прибыль до процентов, налогов и амортизации при продаже, млн ₽</x:v>
       </x:c>
-      <x:c r="B17" s="909" t="n">
+      <x:c r="B17" s="1153" t="n">
         <x:v>2000</x:v>
       </x:c>
       <x:c r="C17" s="90"/>
-      <x:c r="D17" s="1133"/>
-      <x:c r="E17" s="1131"/>
-      <x:c r="F17" s="1132"/>
-      <x:c r="G17" s="1132"/>
-      <x:c r="H17" s="1132"/>
-      <x:c r="I17" s="1132"/>
-      <x:c r="J17" s="1132"/>
-      <x:c r="K17" s="1132"/>
-      <x:c r="L17" s="1132"/>
+      <x:c r="D17" s="1336"/>
+      <x:c r="E17" s="1334"/>
+      <x:c r="F17" s="1335"/>
+      <x:c r="G17" s="1335"/>
+      <x:c r="H17" s="1335"/>
+      <x:c r="I17" s="1335"/>
+      <x:c r="J17" s="1335"/>
+      <x:c r="K17" s="1335"/>
+      <x:c r="L17" s="1335"/>
     </x:row>
     <x:row r="18" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A18" s="3" t="str">
         <x:v>Множитель оценки при продаже, ×</x:v>
       </x:c>
-      <x:c r="B18" s="913" t="n">
+      <x:c r="B18" s="1157" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="89"/>
-      <x:c r="D18" s="1133"/>
-      <x:c r="E18" s="1131"/>
-      <x:c r="F18" s="1132"/>
-      <x:c r="G18" s="1132"/>
-      <x:c r="H18" s="1132"/>
-      <x:c r="I18" s="1132"/>
-      <x:c r="J18" s="1132"/>
-      <x:c r="K18" s="1132"/>
-      <x:c r="L18" s="1132"/>
+      <x:c r="D18" s="1336"/>
+      <x:c r="E18" s="1334"/>
+      <x:c r="F18" s="1335"/>
+      <x:c r="G18" s="1335"/>
+      <x:c r="H18" s="1335"/>
+      <x:c r="I18" s="1335"/>
+      <x:c r="J18" s="1335"/>
+      <x:c r="K18" s="1335"/>
+      <x:c r="L18" s="1335"/>
     </x:row>
     <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A19" t="str">
@@ -4525,67 +5075,67 @@
         <x:v>16000</x:v>
       </x:c>
       <x:c r="C19" s="76"/>
-      <x:c r="D19" s="1134"/>
-      <x:c r="E19" s="1131"/>
-      <x:c r="F19" s="1131"/>
-      <x:c r="G19" s="1131"/>
-      <x:c r="H19" s="1131"/>
-      <x:c r="I19" s="1131"/>
-      <x:c r="J19" s="1131"/>
-      <x:c r="K19" s="1131"/>
-      <x:c r="L19" s="1131"/>
+      <x:c r="D19" s="1337"/>
+      <x:c r="E19" s="1334"/>
+      <x:c r="F19" s="1334"/>
+      <x:c r="G19" s="1334"/>
+      <x:c r="H19" s="1334"/>
+      <x:c r="I19" s="1334"/>
+      <x:c r="J19" s="1334"/>
+      <x:c r="K19" s="1334"/>
+      <x:c r="L19" s="1334"/>
     </x:row>
     <x:row r="20" ht="21.75" customHeight="1">
-      <x:c r="A20" s="907" t="str">
+      <x:c r="A20" s="1151" t="str">
         <x:v>2. Пять ежегодных групп: занятость резерва и закрепление прав к продаже</x:v>
       </x:c>
-      <x:c r="B20" s="907"/>
-      <x:c r="C20" s="907"/>
-      <x:c r="D20" s="907"/>
-      <x:c r="E20" s="907"/>
-      <x:c r="F20" s="907"/>
-      <x:c r="G20" s="907"/>
-      <x:c r="H20" s="907"/>
-      <x:c r="I20" s="907"/>
-      <x:c r="J20" s="907"/>
-      <x:c r="K20" s="907"/>
-      <x:c r="L20" s="907"/>
+      <x:c r="B20" s="1151"/>
+      <x:c r="C20" s="1151"/>
+      <x:c r="D20" s="1151"/>
+      <x:c r="E20" s="1151"/>
+      <x:c r="F20" s="1151"/>
+      <x:c r="G20" s="1151"/>
+      <x:c r="H20" s="1151"/>
+      <x:c r="I20" s="1151"/>
+      <x:c r="J20" s="1151"/>
+      <x:c r="K20" s="1151"/>
+      <x:c r="L20" s="1151"/>
     </x:row>
     <x:row r="21" ht="36" customHeight="1">
-      <x:c r="A21" s="908" t="str">
+      <x:c r="A21" s="1152" t="str">
         <x:v>Год</x:v>
       </x:c>
-      <x:c r="B21" s="908" t="str">
+      <x:c r="B21" s="1152" t="str">
         <x:v>Участников</x:v>
       </x:c>
-      <x:c r="C21" s="908" t="str">
+      <x:c r="C21" s="1152" t="str">
         <x:v>Пакет на человека, млн ₽</x:v>
       </x:c>
-      <x:c r="D21" s="908" t="str">
+      <x:c r="D21" s="1152" t="str">
         <x:v>Пакеты к выдаче, млн ₽</x:v>
       </x:c>
-      <x:c r="E21" s="908" t="str">
+      <x:c r="E21" s="1152" t="str">
         <x:v>Начальная цена единицы, ₽</x:v>
       </x:c>
-      <x:c r="F21" s="908" t="str">
+      <x:c r="F21" s="1152" t="str">
         <x:v>Новые расчётные единицы LTI, млн</x:v>
       </x:c>
-      <x:c r="G21" s="908" t="str">
+      <x:c r="G21" s="1152" t="str">
         <x:v>Занято накопительно, млн</x:v>
       </x:c>
-      <x:c r="H21" s="908" t="str">
+      <x:c r="H21" s="1152" t="str">
         <x:v>Использовано резерва</x:v>
       </x:c>
-      <x:c r="I21" s="908" t="str">
+      <x:c r="I21" s="1152" t="str">
         <x:v>Свободный резерв, млн</x:v>
       </x:c>
-      <x:c r="J21" s="908" t="str">
+      <x:c r="J21" s="1152" t="str">
         <x:v>Закрепилось к продаже</x:v>
       </x:c>
-      <x:c r="K21" s="908" t="str">
+      <x:c r="K21" s="1152" t="str">
         <x:v>Закрепившиеся расчётные единицы, млн</x:v>
       </x:c>
-      <x:c r="L21" s="908" t="str">
+      <x:c r="L21" s="1152" t="str">
         <x:v>Валовая стоимость при продаже, млн ₽</x:v>
       </x:c>
     </x:row>
@@ -4593,17 +5143,16 @@
       <x:c r="A22" s="3" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B22" s="287" t="n">
-        <x:f>$B$12</x:f>
-        <x:v>15</x:v>
+      <x:c r="B22" s="1154" t="n">
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="275" t="n">
         <x:f>$B$15</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D22" s="275" t="n">
-        <x:f>$B$16</x:f>
-        <x:v>52.5</x:v>
+        <x:f>B22*C22</x:f>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E22" s="275" t="n">
         <x:f>I10</x:f>
@@ -4611,47 +5160,46 @@
       </x:c>
       <x:c r="F22" s="275" t="n">
         <x:f>D22/E22</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="G22" s="275" t="n">
         <x:f>SUM($F$22:F22)</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="H22" s="279" t="n">
         <x:f>G22/$B$11</x:f>
-        <x:v>0.4375</x:v>
+        <x:v>0.33333333333333337</x:v>
       </x:c>
       <x:c r="I22" s="275" t="n">
         <x:f>$B$11-G22</x:f>
-        <x:v>5.625</x:v>
+        <x:v>6.666666666666666</x:v>
       </x:c>
       <x:c r="J22" s="279" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K22" s="275" t="n">
         <x:f>F22*J22</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="L22" s="290" t="n">
         <x:f>K22*($B$19/$K$14)</x:f>
-        <x:v>340.50203990594486</x:v>
+        <x:v>259.43012564262466</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="21.75" customHeight="1">
       <x:c r="A23" s="8" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B23" s="287" t="n">
-        <x:f>$B$12</x:f>
-        <x:v>15</x:v>
+      <x:c r="B23" s="1154" t="n">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C23" s="275" t="n">
         <x:f>$B$15</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D23" s="275" t="n">
-        <x:f>$B$16</x:f>
-        <x:v>52.5</x:v>
+        <x:f>B23*C23</x:f>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E23" s="275" t="n">
         <x:f>I11</x:f>
@@ -4659,47 +5207,46 @@
       </x:c>
       <x:c r="F23" s="275" t="n">
         <x:f>D23/E23</x:f>
-        <x:v>2.1875</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="G23" s="275" t="n">
         <x:f>SUM($F$22:F23)</x:f>
-        <x:v>6.5625</x:v>
+        <x:v>5.833333333333334</x:v>
       </x:c>
       <x:c r="H23" s="279" t="n">
         <x:f>G23/$B$11</x:f>
-        <x:v>0.65625</x:v>
+        <x:v>0.5833333333333334</x:v>
       </x:c>
       <x:c r="I23" s="275" t="n">
         <x:f>$B$11-G23</x:f>
-        <x:v>3.4375</x:v>
+        <x:v>4.166666666666666</x:v>
       </x:c>
       <x:c r="J23" s="279" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="K23" s="275" t="n">
         <x:f>F23*J23</x:f>
-        <x:v>2.1875</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="L23" s="276" t="n">
         <x:f>K23*($B$19/$K$14)</x:f>
-        <x:v>170.25101995297243</x:v>
+        <x:v>194.57259423196848</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="21.75" customHeight="1">
       <x:c r="A24" s="3" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B24" s="287" t="n">
-        <x:f>$B$12</x:f>
-        <x:v>15</x:v>
+      <x:c r="B24" s="1154" t="n">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C24" s="275" t="n">
         <x:f>$B$15</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D24" s="275" t="n">
-        <x:f>$B$16</x:f>
-        <x:v>52.5</x:v>
+        <x:f>B24*C24</x:f>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E24" s="275" t="n">
         <x:f>I12</x:f>
@@ -4707,19 +5254,19 @@
       </x:c>
       <x:c r="F24" s="275" t="n">
         <x:f>D24/E24</x:f>
-        <x:v>1.3671875</x:v>
+        <x:v>1.5625</x:v>
       </x:c>
       <x:c r="G24" s="275" t="n">
         <x:f>SUM($F$22:F24)</x:f>
-        <x:v>7.9296875</x:v>
+        <x:v>7.395833333333334</x:v>
       </x:c>
       <x:c r="H24" s="279" t="n">
         <x:f>G24/$B$11</x:f>
-        <x:v>0.79296875</x:v>
+        <x:v>0.7395833333333334</x:v>
       </x:c>
       <x:c r="I24" s="275" t="n">
         <x:f>$B$11-G24</x:f>
-        <x:v>2.0703125</x:v>
+        <x:v>2.604166666666666</x:v>
       </x:c>
       <x:c r="J24" s="279" t="n">
         <x:f>2/3</x:f>
@@ -4727,28 +5274,27 @@
       </x:c>
       <x:c r="K24" s="275" t="n">
         <x:f>F24*J24</x:f>
-        <x:v>0.9114583333333333</x:v>
+        <x:v>1.0416666666666665</x:v>
       </x:c>
       <x:c r="L24" s="290" t="n">
         <x:f>K24*($B$19/$K$14)</x:f>
-        <x:v>70.93792498040517</x:v>
+        <x:v>81.0719142633202</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="21.75" customHeight="1">
       <x:c r="A25" s="8" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B25" s="287" t="n">
-        <x:f>$B$12</x:f>
-        <x:v>15</x:v>
+      <x:c r="B25" s="1154" t="n">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C25" s="275" t="n">
         <x:f>$B$15</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D25" s="275" t="n">
-        <x:f>$B$16</x:f>
-        <x:v>52.5</x:v>
+        <x:f>B25*C25</x:f>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E25" s="275" t="n">
         <x:f>I13</x:f>
@@ -4756,19 +5302,19 @@
       </x:c>
       <x:c r="F25" s="275" t="n">
         <x:f>D25/E25</x:f>
-        <x:v>0.9435017903645834</x:v>
+        <x:v>1.0782877604166667</x:v>
       </x:c>
       <x:c r="G25" s="275" t="n">
         <x:f>SUM($F$22:F25)</x:f>
-        <x:v>8.873189290364584</x:v>
+        <x:v>8.47412109375</x:v>
       </x:c>
       <x:c r="H25" s="279" t="n">
         <x:f>G25/$B$11</x:f>
-        <x:v>0.8873189290364584</x:v>
+        <x:v>0.847412109375</x:v>
       </x:c>
       <x:c r="I25" s="275" t="n">
         <x:f>$B$11-G25</x:f>
-        <x:v>1.126810709635416</x:v>
+        <x:v>1.52587890625</x:v>
       </x:c>
       <x:c r="J25" s="279" t="n">
         <x:f>1/3</x:f>
@@ -4776,28 +5322,27 @@
       </x:c>
       <x:c r="K25" s="275" t="n">
         <x:f>F25*J25</x:f>
-        <x:v>0.3145005967881944</x:v>
+        <x:v>0.3594292534722222</x:v>
       </x:c>
       <x:c r="L25" s="276" t="n">
         <x:f>K25*($B$19/$K$14)</x:f>
-        <x:v>24.477278801832515</x:v>
+        <x:v>27.97403291638002</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="21.75" customHeight="1">
       <x:c r="A26" s="3" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B26" s="288" t="n">
-        <x:f>$B$12</x:f>
+      <x:c r="B26" s="1154" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="C26" s="290" t="n">
         <x:f>$B$15</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D26" s="290" t="n">
-        <x:f>$B$16</x:f>
-        <x:v>52.5</x:v>
+        <x:f>B26*C26</x:f>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="E26" s="290" t="n">
         <x:f>I14</x:f>
@@ -4805,19 +5350,19 @@
       </x:c>
       <x:c r="F26" s="290" t="n">
         <x:f>D26/E26</x:f>
-        <x:v>0.7212953701482118</x:v>
+        <x:v>1.0304219573545883</x:v>
       </x:c>
       <x:c r="G26" s="290" t="n">
         <x:f>SUM($F$22:F26)</x:f>
-        <x:v>9.594484660512796</x:v>
+        <x:v>9.504543051104589</x:v>
       </x:c>
       <x:c r="H26" s="292" t="n">
         <x:f>G26/$B$11</x:f>
-        <x:v>0.9594484660512796</x:v>
+        <x:v>0.9504543051104589</x:v>
       </x:c>
       <x:c r="I26" s="290" t="n">
         <x:f>$B$11-G26</x:f>
-        <x:v>0.405515339487204</x:v>
+        <x:v>0.49545694889541103</x:v>
       </x:c>
       <x:c r="J26" s="292" t="n">
         <x:v>0</x:v>
@@ -4832,78 +5377,78 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="926" t="str">
+      <x:c r="A27" s="1171" t="str">
         <x:v>ИТОГО</x:v>
       </x:c>
-      <x:c r="B27" s="931" t="n">
+      <x:c r="B27" s="1176" t="n">
         <x:f>SUM(B22:B26)</x:f>
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="C27" s="932" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C27" s="1177" t="n">
         <x:f>AVERAGE(C22:C26)</x:f>
-        <x:v>3.5</x:v>
-      </x:c>
-      <x:c r="D27" s="932" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D27" s="1177" t="n">
         <x:f>SUM(D22:D26)</x:f>
-        <x:v>262.5</x:v>
-      </x:c>
-      <x:c r="E27" s="932"/>
-      <x:c r="F27" s="932" t="n">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="E27" s="1177"/>
+      <x:c r="F27" s="1177" t="n">
         <x:f>SUM(F22:F26)</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="G27" s="932" t="n">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="G27" s="1177" t="n">
         <x:f>MAX(G22:G26)</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="H27" s="933" t="n">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="H27" s="1178" t="n">
         <x:f>MAX(H22:H26)</x:f>
-        <x:v>0.9594484660512796</x:v>
-      </x:c>
-      <x:c r="I27" s="932" t="n">
+        <x:v>0.9504543051104589</x:v>
+      </x:c>
+      <x:c r="I27" s="1177" t="n">
         <x:f>$B$11-G27</x:f>
-        <x:v>0.405515339487204</x:v>
-      </x:c>
-      <x:c r="J27" s="926"/>
-      <x:c r="K27" s="932" t="n">
+        <x:v>0.49545694889541103</x:v>
+      </x:c>
+      <x:c r="J27" s="1171"/>
+      <x:c r="K27" s="1177" t="n">
         <x:f>SUM(K22:K26)</x:f>
-        <x:v>7.788458930121528</x:v>
-      </x:c>
-      <x:c r="L27" s="932" t="n">
+        <x:v>7.234429253472222</x:v>
+      </x:c>
+      <x:c r="L27" s="1177" t="n">
         <x:f>SUM(L22:L26)</x:f>
-        <x:v>606.168263641155</x:v>
+        <x:v>563.0486670542933</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="21.75" customHeight="1">
-      <x:c r="A28" s="907" t="str">
+      <x:c r="A28" s="1151" t="str">
         <x:v>3. Что именно существует к продаже после пятого года</x:v>
       </x:c>
-      <x:c r="B28" s="907"/>
-      <x:c r="C28" s="907"/>
-      <x:c r="D28" s="907"/>
-      <x:c r="E28" s="907"/>
-      <x:c r="F28" s="907"/>
-      <x:c r="G28" s="907"/>
-      <x:c r="H28" s="907"/>
-      <x:c r="I28" s="907"/>
-      <x:c r="J28" s="907"/>
-      <x:c r="K28" s="907"/>
-      <x:c r="L28" s="907"/>
+      <x:c r="B28" s="1151"/>
+      <x:c r="C28" s="1151"/>
+      <x:c r="D28" s="1151"/>
+      <x:c r="E28" s="1151"/>
+      <x:c r="F28" s="1151"/>
+      <x:c r="G28" s="1151"/>
+      <x:c r="H28" s="1151"/>
+      <x:c r="I28" s="1151"/>
+      <x:c r="J28" s="1151"/>
+      <x:c r="K28" s="1151"/>
+      <x:c r="L28" s="1151"/>
     </x:row>
     <x:row r="29" ht="31.5" customHeight="1">
-      <x:c r="A29" s="908" t="str">
+      <x:c r="A29" s="1152" t="str">
         <x:v>Показатель</x:v>
       </x:c>
-      <x:c r="B29" s="908" t="str">
+      <x:c r="B29" s="1152" t="str">
         <x:v>Единиц, млн</x:v>
       </x:c>
-      <x:c r="C29" s="908" t="str">
+      <x:c r="C29" s="1152" t="str">
         <x:v>Доля компании</x:v>
       </x:c>
-      <x:c r="D29" s="908" t="str">
+      <x:c r="D29" s="1152" t="str">
         <x:v>Стоимость при продаже, млн ₽</x:v>
       </x:c>
-      <x:c r="E29" s="908" t="str">
+      <x:c r="E29" s="1152" t="str">
         <x:v>Смысл</x:v>
       </x:c>
       <x:c r="F29" s="2"/>
@@ -4947,15 +5492,15 @@
       </x:c>
       <x:c r="B31" s="303" t="n">
         <x:f>$G$27</x:f>
-        <x:v>9.594484660512796</x:v>
+        <x:v>9.504543051104589</x:v>
       </x:c>
       <x:c r="C31" s="307" t="n">
         <x:f>B31/$K$14</x:f>
-        <x:v>0.046670594267870055</x:v>
+        <x:v>0.04623308996107122</x:v>
       </x:c>
       <x:c r="D31" s="311" t="n">
         <x:f>B31*($B$19/$K$14)</x:f>
-        <x:v>746.7295082859209</x:v>
+        <x:v>739.7294393771396</x:v>
       </x:c>
       <x:c r="E31" s="20" t="str">
         <x:v>Включает ещё не закрепившуюся часть последних пакетов</x:v>
@@ -4969,22 +5514,22 @@
       <x:c r="L31" s="17"/>
     </x:row>
     <x:row r="32" ht="28.5" customHeight="1">
-      <x:c r="A32" s="934" t="str">
+      <x:c r="A32" s="1179" t="str">
         <x:v>Закрепилось к продаже</x:v>
       </x:c>
-      <x:c r="B32" s="935" t="n">
+      <x:c r="B32" s="1180" t="n">
         <x:f>$K$27</x:f>
-        <x:v>7.788458930121528</x:v>
-      </x:c>
-      <x:c r="C32" s="936" t="n">
+        <x:v>7.234429253472222</x:v>
+      </x:c>
+      <x:c r="C32" s="1181" t="n">
         <x:f>B32/$K$14</x:f>
-        <x:v>0.037885516477572184</x:v>
-      </x:c>
-      <x:c r="D32" s="937" t="n">
+        <x:v>0.035190541690893334</x:v>
+      </x:c>
+      <x:c r="D32" s="1182" t="n">
         <x:f>$L$27</x:f>
-        <x:v>606.168263641155</x:v>
-      </x:c>
-      <x:c r="E32" s="938" t="str">
+        <x:v>563.0486670542933</x:v>
+      </x:c>
+      <x:c r="E32" s="1183" t="str">
         <x:v>Эта часть участвует в расчёте валовой стоимости</x:v>
       </x:c>
       <x:c r="F32" s="13"/>
@@ -4996,22 +5541,22 @@
       <x:c r="L32" s="3"/>
     </x:row>
     <x:row r="33" ht="28.5" customHeight="1">
-      <x:c r="A33" s="939" t="str">
+      <x:c r="A33" s="1184" t="str">
         <x:v>Не закрепилось к продаже</x:v>
       </x:c>
-      <x:c r="B33" s="940" t="n">
+      <x:c r="B33" s="1185" t="n">
         <x:f>B31-B32</x:f>
-        <x:v>1.8060257303912683</x:v>
-      </x:c>
-      <x:c r="C33" s="941" t="n">
+        <x:v>2.2701137976323666</x:v>
+      </x:c>
+      <x:c r="C33" s="1186" t="n">
         <x:f>B33/$K$14</x:f>
-        <x:v>0.00878507779029787</x:v>
-      </x:c>
-      <x:c r="D33" s="942" t="n">
+        <x:v>0.011042548270177886</x:v>
+      </x:c>
+      <x:c r="D33" s="1187" t="n">
         <x:f>B33*($B$19/$K$14)</x:f>
-        <x:v>140.5612446447659</x:v>
-      </x:c>
-      <x:c r="E33" s="943" t="str">
+        <x:v>176.6807723228462</x:v>
+      </x:c>
+      <x:c r="E33" s="1188" t="str">
         <x:v>Для поздних пакетов 36 месяцев ещё не прошли</x:v>
       </x:c>
     </x:row>
@@ -5030,35 +5575,35 @@
       <x:c r="L34" s="27"/>
     </x:row>
     <x:row r="35" ht="21.75" customHeight="1">
-      <x:c r="A35" s="907" t="str">
+      <x:c r="A35" s="1151" t="str">
         <x:v>4. Контрольные проверки</x:v>
       </x:c>
-      <x:c r="B35" s="907"/>
-      <x:c r="C35" s="907"/>
-      <x:c r="D35" s="907"/>
-      <x:c r="E35" s="907"/>
-      <x:c r="F35" s="907"/>
-      <x:c r="G35" s="907"/>
-      <x:c r="H35" s="907"/>
-      <x:c r="I35" s="907"/>
-      <x:c r="J35" s="907"/>
-      <x:c r="K35" s="907"/>
-      <x:c r="L35" s="907"/>
+      <x:c r="B35" s="1151"/>
+      <x:c r="C35" s="1151"/>
+      <x:c r="D35" s="1151"/>
+      <x:c r="E35" s="1151"/>
+      <x:c r="F35" s="1151"/>
+      <x:c r="G35" s="1151"/>
+      <x:c r="H35" s="1151"/>
+      <x:c r="I35" s="1151"/>
+      <x:c r="J35" s="1151"/>
+      <x:c r="K35" s="1151"/>
+      <x:c r="L35" s="1151"/>
     </x:row>
     <x:row r="36" ht="36" customHeight="1">
-      <x:c r="A36" s="908" t="str">
+      <x:c r="A36" s="1152" t="str">
         <x:v>Проверка</x:v>
       </x:c>
-      <x:c r="B36" s="908" t="str">
+      <x:c r="B36" s="1152" t="str">
         <x:v>Факт</x:v>
       </x:c>
-      <x:c r="C36" s="908" t="str">
+      <x:c r="C36" s="1152" t="str">
         <x:v>Ожидается / предел</x:v>
       </x:c>
-      <x:c r="D36" s="908" t="str">
+      <x:c r="D36" s="1152" t="str">
         <x:v>Отклонение</x:v>
       </x:c>
-      <x:c r="E36" s="908" t="str">
+      <x:c r="E36" s="1152" t="str">
         <x:v>Статус</x:v>
       </x:c>
       <x:c r="F36" s="2"/>
@@ -5175,7 +5720,7 @@
       </x:c>
       <x:c r="B40" s="275" t="n">
         <x:f>$G$27</x:f>
-        <x:v>9.594484660512796</x:v>
+        <x:v>9.504543051104589</x:v>
       </x:c>
       <x:c r="C40" s="290" t="n">
         <x:f>$B$11</x:f>
@@ -5183,7 +5728,7 @@
       </x:c>
       <x:c r="D40" s="290" t="n">
         <x:f>B40-C40</x:f>
-        <x:v>-0.405515339487204</x:v>
+        <x:v>-0.49545694889541103</x:v>
       </x:c>
       <x:c r="E40" s="292" t="str">
         <x:f>IF(B40&lt;=C40,"НОРМА","СТОП")</x:f>
@@ -5209,14 +5754,14 @@
       </x:c>
       <x:c r="B41" s="275" t="n">
         <x:f>$I$27</x:f>
-        <x:v>0.405515339487204</x:v>
+        <x:v>0.49545694889541103</x:v>
       </x:c>
       <x:c r="C41" s="276" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D41" s="276" t="n">
         <x:f>B41-C41</x:f>
-        <x:v>0.405515339487204</x:v>
+        <x:v>0.49545694889541103</x:v>
       </x:c>
       <x:c r="E41" s="315" t="str">
         <x:f>IF(B41&gt;=C41,"НОРМА","СТОП")</x:f>
@@ -5237,13 +5782,13 @@
       </x:c>
     </x:row>
     <x:row r="42" ht="21.75" customHeight="1">
-      <x:c r="A42" s="944" t="str">
+      <x:c r="A42" s="1189" t="str">
         <x:v>СТАТУС МОДЕЛИ</x:v>
       </x:c>
-      <x:c r="B42" s="944"/>
-      <x:c r="C42" s="948"/>
-      <x:c r="D42" s="948"/>
-      <x:c r="E42" s="949" t="str">
+      <x:c r="B42" s="1189"/>
+      <x:c r="C42" s="1193"/>
+      <x:c r="D42" s="1193"/>
+      <x:c r="E42" s="1194" t="str">
         <x:f>IF(COUNTIF(E37:E41,"&lt;&gt;НОРМА")=0,"ПРОЙДЕНО","ПРОВЕРИТЬ")</x:f>
         <x:v>ПРОЙДЕНО</x:v>
       </x:c>
@@ -5262,24 +5807,24 @@
       </x:c>
     </x:row>
     <x:row r="44" ht="21.75" customHeight="1">
-      <x:c r="A44" s="907" t="str">
+      <x:c r="A44" s="1151" t="str">
         <x:v>5. Как читать модель</x:v>
       </x:c>
-      <x:c r="B44" s="907"/>
-      <x:c r="C44" s="907"/>
-      <x:c r="D44" s="907"/>
-      <x:c r="E44" s="907"/>
-      <x:c r="F44" s="907"/>
-      <x:c r="G44" s="907"/>
-      <x:c r="H44" s="907"/>
-      <x:c r="I44" s="907"/>
-      <x:c r="J44" s="907"/>
-      <x:c r="K44" s="907"/>
-      <x:c r="L44" s="907"/>
+      <x:c r="B44" s="1151"/>
+      <x:c r="C44" s="1151"/>
+      <x:c r="D44" s="1151"/>
+      <x:c r="E44" s="1151"/>
+      <x:c r="F44" s="1151"/>
+      <x:c r="G44" s="1151"/>
+      <x:c r="H44" s="1151"/>
+      <x:c r="I44" s="1151"/>
+      <x:c r="J44" s="1151"/>
+      <x:c r="K44" s="1151"/>
+      <x:c r="L44" s="1151"/>
     </x:row>
     <x:row r="45" ht="22.5" customHeight="1">
       <x:c r="A45" s="323" t="str">
-        <x:v>1. Каждый год Совет отдельно выбирает 15 участников; средний пакет в примере равен 0,7 годового оклада, или 3,5 млн ₽ на человека.</x:v>
+        <x:v>1. Совет выбирает 8 участников в первый год, до 12 в годы 2–4 и до 15 в пятом году как резерв максимального расширения. Ёмкость проверяется по максимальному пакету 1,0 оклада, или 5 млн ₽.</x:v>
       </x:c>
       <x:c r="B45" s="323"/>
       <x:c r="C45" s="323"/>
@@ -5358,20 +5903,20 @@
       <x:c r="L49" s="76"/>
     </x:row>
     <x:row r="50" ht="33" customHeight="1">
-      <x:c r="A50" s="950" t="str">
+      <x:c r="A50" s="1195" t="str">
         <x:v>Все суммы — валовые до налогов, долга, расходов и порядка распределения выплат. Это управленческая модель, а не обещание выплаты. Расчёты соответствуют модели сайта.</x:v>
       </x:c>
-      <x:c r="B50" s="950"/>
-      <x:c r="C50" s="950"/>
-      <x:c r="D50" s="950"/>
-      <x:c r="E50" s="950"/>
-      <x:c r="F50" s="950"/>
-      <x:c r="G50" s="950"/>
-      <x:c r="H50" s="950"/>
-      <x:c r="I50" s="950"/>
-      <x:c r="J50" s="950"/>
-      <x:c r="K50" s="950"/>
-      <x:c r="L50" s="950"/>
+      <x:c r="B50" s="1195"/>
+      <x:c r="C50" s="1195"/>
+      <x:c r="D50" s="1195"/>
+      <x:c r="E50" s="1195"/>
+      <x:c r="F50" s="1195"/>
+      <x:c r="G50" s="1195"/>
+      <x:c r="H50" s="1195"/>
+      <x:c r="I50" s="1195"/>
+      <x:c r="J50" s="1195"/>
+      <x:c r="K50" s="1195"/>
+      <x:c r="L50" s="1195"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -5437,7 +5982,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb20c8e671f914346"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b001ef0c4b64877"/>
 </x:worksheet>
 </file>
 
@@ -5456,7 +6001,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="A1" s="898" t="str">
+      <x:c r="A1" s="1142" t="str">
         <x:v>Личный пример: пять ежегодных пакетов и продажа после пятого года</x:v>
       </x:c>
       <x:c r="B1" s="56"/>
@@ -5468,38 +6013,38 @@
       <x:c r="H1" s="56"/>
     </x:row>
     <x:row r="2" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A2" s="951" t="str">
+      <x:c r="A2" s="1196" t="str">
         <x:v>Закрепление права — постепенный переход уже заработанного пакета: 1/12 каждые три месяца в течение 36 месяцев после годового подтверждения результата.</x:v>
       </x:c>
-      <x:c r="B2" s="951"/>
-      <x:c r="C2" s="951"/>
-      <x:c r="D2" s="951"/>
-      <x:c r="E2" s="951"/>
-      <x:c r="F2" s="951"/>
-      <x:c r="G2" s="951"/>
-      <x:c r="H2" s="951"/>
+      <x:c r="B2" s="1196"/>
+      <x:c r="C2" s="1196"/>
+      <x:c r="D2" s="1196"/>
+      <x:c r="E2" s="1196"/>
+      <x:c r="F2" s="1196"/>
+      <x:c r="G2" s="1196"/>
+      <x:c r="H2" s="1196"/>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="36" hidden="0" customHeight="1">
-      <x:c r="A4" s="914" t="str">
+      <x:c r="A4" s="1158" t="str">
         <x:v>Общие допущения</x:v>
       </x:c>
-      <x:c r="B4" s="914" t="str">
+      <x:c r="B4" s="1158" t="str">
         <x:v>Значение</x:v>
       </x:c>
-      <x:c r="D4" s="914" t="str">
+      <x:c r="D4" s="1158" t="str">
         <x:v>Год</x:v>
       </x:c>
-      <x:c r="E4" s="914" t="str">
+      <x:c r="E4" s="1158" t="str">
         <x:v>Начальная цена, ₽</x:v>
       </x:c>
-      <x:c r="F4" s="914" t="str">
+      <x:c r="F4" s="1158" t="str">
         <x:v>Расчётных единиц пакета, млн</x:v>
       </x:c>
-      <x:c r="G4" s="914" t="str">
+      <x:c r="G4" s="1158" t="str">
         <x:v>Закрепилось к продаже</x:v>
       </x:c>
-      <x:c r="H4" s="914" t="str">
+      <x:c r="H4" s="1158" t="str">
         <x:v>Валовая стоимость, млн ₽</x:v>
       </x:c>
     </x:row>
@@ -5519,8 +6064,8 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="F5" s="353" t="n">
-        <x:f>$B$7/E5</x:f>
-        <x:v>0.2916666666666667</x:v>
+        <x:f>$B$8/E5</x:f>
+        <x:v>0.3958333333333333</x:v>
       </x:c>
       <x:c r="G5" s="354" t="n">
         <x:f>'Калькулятор'!J22</x:f>
@@ -5528,16 +6073,16 @@
       </x:c>
       <x:c r="H5" s="243" t="n">
         <x:f>F5*G5*$B$10</x:f>
-        <x:v>22.70013599372966</x:v>
+        <x:v>30.807327420061675</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="76" t="str">
-        <x:v>Средний множитель пакета, ×</x:v>
+        <x:v>Целевой множитель пакета, ×</x:v>
       </x:c>
       <x:c r="B6" s="338" t="n">
         <x:f>'Калькулятор'!B14</x:f>
-        <x:v>0.7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D6" s="76" t="n">
         <x:v>2</x:v>
@@ -5547,8 +6092,8 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="F6" s="353" t="n">
-        <x:f>$B$7/E6</x:f>
-        <x:v>0.14583333333333334</x:v>
+        <x:f>$B$8/E6</x:f>
+        <x:v>0.19791666666666666</x:v>
       </x:c>
       <x:c r="G6" s="354" t="n">
         <x:f>'Калькулятор'!J23</x:f>
@@ -5556,16 +6101,15 @@
       </x:c>
       <x:c r="H6" s="243" t="n">
         <x:f>F6*G6*$B$10</x:f>
-        <x:v>11.35006799686483</x:v>
+        <x:v>15.403663710030838</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="76" t="str">
-        <x:v>Пакет на год, млн ₽</x:v>
-      </x:c>
-      <x:c r="B7" s="339" t="n">
-        <x:f>B5*B6</x:f>
-        <x:v>3.5</x:v>
+        <x:v>Подтверждённый результат</x:v>
+      </x:c>
+      <x:c r="B7" s="1199" t="n">
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="D7" s="76" t="n">
         <x:v>3</x:v>
@@ -5575,8 +6119,8 @@
         <x:v>38.4</x:v>
       </x:c>
       <x:c r="F7" s="353" t="n">
-        <x:f>$B$7/E7</x:f>
-        <x:v>0.09114583333333334</x:v>
+        <x:f>$B$8/E7</x:f>
+        <x:v>0.12369791666666667</x:v>
       </x:c>
       <x:c r="G7" s="354" t="n">
         <x:f>'Калькулятор'!J24</x:f>
@@ -5584,16 +6128,16 @@
       </x:c>
       <x:c r="H7" s="243" t="n">
         <x:f>F7*G7*$B$10</x:f>
-        <x:v>4.729194998693679</x:v>
+        <x:v>6.41819321251285</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="76" t="str">
-        <x:v>Стоимость капитала при продаже, млн ₽</x:v>
-      </x:c>
-      <x:c r="B8" s="337" t="n">
-        <x:f>'Калькулятор'!B19</x:f>
-        <x:v>16000</x:v>
+        <x:v>Заработанный пакет на год, млн ₽</x:v>
+      </x:c>
+      <x:c r="B8" s="341" t="n">
+        <x:f>B5*B6*B7</x:f>
+        <x:v>4.75</x:v>
       </x:c>
       <x:c r="D8" s="76" t="n">
         <x:v>4</x:v>
@@ -5603,8 +6147,8 @@
         <x:v>55.64377358490566</x:v>
       </x:c>
       <x:c r="F8" s="353" t="n">
-        <x:f>$B$7/E8</x:f>
-        <x:v>0.0629001193576389</x:v>
+        <x:f>$B$8/E8</x:f>
+        <x:v>0.08536444769965278</x:v>
       </x:c>
       <x:c r="G8" s="354" t="n">
         <x:f>'Калькулятор'!J25</x:f>
@@ -5612,7 +6156,7 @@
       </x:c>
       <x:c r="H8" s="243" t="n">
         <x:f>F8*G8*$B$10</x:f>
-        <x:v>1.6318185867888344</x:v>
+        <x:v>2.214610939213418</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -5631,8 +6175,8 @@
         <x:v>72.78571605029477</x:v>
       </x:c>
       <x:c r="F9" s="353" t="n">
-        <x:f>$B$7/E9</x:f>
-        <x:v>0.04808635800988078</x:v>
+        <x:f>$B$8/E9</x:f>
+        <x:v>0.06526005729912392</x:v>
       </x:c>
       <x:c r="G9" s="354" t="n">
         <x:f>'Калькулятор'!J26</x:f>
@@ -5648,21 +6192,21 @@
         <x:v>Цена расчётной единицы при продаже, ₽</x:v>
       </x:c>
       <x:c r="B10" s="341" t="n">
-        <x:f>B8/B9</x:f>
+        <x:f>'Калькулятор'!B19/B9</x:f>
         <x:v>77.8290376927874</x:v>
       </x:c>
-      <x:c r="D10" s="952" t="str">
+      <x:c r="D10" s="1200" t="str">
         <x:v>ИТОГО</x:v>
       </x:c>
-      <x:c r="E10" s="952"/>
-      <x:c r="F10" s="932" t="n">
+      <x:c r="E10" s="1200"/>
+      <x:c r="F10" s="1177" t="n">
         <x:f>SUM(F5:F9)</x:f>
-        <x:v>0.6396323107008531</x:v>
-      </x:c>
-      <x:c r="G10" s="926"/>
-      <x:c r="H10" s="917" t="n">
+        <x:v>0.8680724216654433</x:v>
+      </x:c>
+      <x:c r="G10" s="1171"/>
+      <x:c r="H10" s="1161" t="n">
         <x:f>SUM(H5:H9)</x:f>
-        <x:v>40.411217576077</x:v>
+        <x:v>54.84379528181877</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -5673,19 +6217,19 @@
       <x:c r="F11" s="84"/>
     </x:row>
     <x:row r="12" ht="22.5" hidden="0" customHeight="1">
-      <x:c r="A12" s="914" t="str">
+      <x:c r="A12" s="1158" t="str">
         <x:v>Итог личного примера</x:v>
       </x:c>
-      <x:c r="B12" s="954" t="str">
+      <x:c r="B12" s="1202" t="str">
         <x:v>Значение</x:v>
       </x:c>
-      <x:c r="D12" s="956" t="str">
+      <x:c r="D12" s="1204" t="str">
         <x:v>Почему не вся сумма закрепилась</x:v>
       </x:c>
-      <x:c r="E12" s="956"/>
-      <x:c r="F12" s="957"/>
-      <x:c r="G12" s="958"/>
-      <x:c r="H12" s="958"/>
+      <x:c r="E12" s="1204"/>
+      <x:c r="F12" s="1205"/>
+      <x:c r="G12" s="1206"/>
+      <x:c r="H12" s="1206"/>
     </x:row>
     <x:row r="13" ht="25.5" hidden="0" customHeight="1">
       <x:c r="A13" s="76" t="str">
@@ -5693,7 +6237,7 @@
       </x:c>
       <x:c r="B13" s="339" t="n">
         <x:f>SUM(F5:F9)*B10</x:f>
-        <x:v>49.7819672190614</x:v>
+        <x:v>67.56124122586903</x:v>
       </x:c>
       <x:c r="D13" s="76" t="str">
         <x:v>Пакеты лет 1–2 к продаже прошли все 36 месяцев.</x:v>
@@ -5704,12 +6248,12 @@
       <x:c r="H13" s="76"/>
     </x:row>
     <x:row r="14" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="A14" s="952" t="str">
+      <x:c r="A14" s="1200" t="str">
         <x:v>Закрепившаяся стоимость, млн ₽</x:v>
       </x:c>
-      <x:c r="B14" s="917" t="n">
+      <x:c r="B14" s="1161" t="n">
         <x:f>SUM(H5:H9)</x:f>
-        <x:v>40.411217576077</x:v>
+        <x:v>54.84379528181877</x:v>
       </x:c>
       <x:c r="D14" s="76" t="str">
         <x:v>Пакет года 3 закрепился на 2/3, года 4 — на 1/3.</x:v>
@@ -5720,12 +6264,12 @@
       <x:c r="H14" s="76"/>
     </x:row>
     <x:row r="15" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="A15" s="943" t="str">
+      <x:c r="A15" s="1188" t="str">
         <x:v>Незакрепившаяся стоимость, млн ₽</x:v>
       </x:c>
-      <x:c r="B15" s="955" t="n">
+      <x:c r="B15" s="1203" t="n">
         <x:f>B13-B14</x:f>
-        <x:v>9.3707496429844</x:v>
+        <x:v>12.717445944050255</x:v>
       </x:c>
       <x:c r="D15" s="76" t="str">
         <x:v>Пакет года 5 только подтверждён и ещё не начал закрепляться.</x:v>
@@ -5741,7 +6285,7 @@
       </x:c>
       <x:c r="B16" s="367" t="n">
         <x:f>F5*G5+F6*G6+F7*G7+F8*G8+F9*G9</x:f>
-        <x:v>0.5192305953414352</x:v>
+        <x:v>0.7046700936776621</x:v>
       </x:c>
       <x:c r="D16" s="76" t="str">
         <x:v>Незакрепившаяся часть не включена в показанную валовую стоимость.</x:v>
@@ -5754,31 +6298,31 @@
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="76"/>
       <x:c r="B17" s="79"/>
-      <x:c r="D17" s="1131"/>
-      <x:c r="E17" s="1131"/>
-      <x:c r="F17" s="1131"/>
-      <x:c r="G17" s="1131"/>
-      <x:c r="H17" s="1131"/>
+      <x:c r="D17" s="1334"/>
+      <x:c r="E17" s="1334"/>
+      <x:c r="F17" s="1334"/>
+      <x:c r="G17" s="1334"/>
+      <x:c r="H17" s="1334"/>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="76"/>
       <x:c r="B18" s="65"/>
-      <x:c r="D18" s="1131"/>
-      <x:c r="E18" s="1135"/>
-      <x:c r="F18" s="1135"/>
-      <x:c r="G18" s="1135"/>
-      <x:c r="H18" s="1135"/>
+      <x:c r="D18" s="1334"/>
+      <x:c r="E18" s="1338"/>
+      <x:c r="F18" s="1338"/>
+      <x:c r="G18" s="1338"/>
+      <x:c r="H18" s="1338"/>
     </x:row>
     <x:row r="19"/>
     <x:row r="20" ht="22.5" hidden="0" customHeight="1">
-      <x:c r="A20" s="914" t="str">
+      <x:c r="A20" s="1158" t="str">
         <x:v>Момент</x:v>
       </x:c>
-      <x:c r="B20" s="914" t="str">
+      <x:c r="B20" s="1158" t="str">
         <x:v>Что происходит</x:v>
       </x:c>
-      <x:c r="C20" s="914"/>
-      <x:c r="D20" s="914" t="str">
+      <x:c r="C20" s="1158"/>
+      <x:c r="D20" s="1158" t="str">
         <x:v>Состояние прав</x:v>
       </x:c>
       <x:c r="E20" s="75"/>
@@ -5803,11 +6347,11 @@
         <x:v>Конец года</x:v>
       </x:c>
       <x:c r="B22" s="101" t="str">
-        <x:v>Совет подтверждает результат и число расчётных единиц</x:v>
+        <x:v>После итогового расчёта начинается закрепление права</x:v>
       </x:c>
       <x:c r="C22" s="101"/>
       <x:c r="D22" s="101" t="str">
-        <x:v>Начало закрепления права</x:v>
+        <x:v>По 1/12 за полный квартал</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="28.5" hidden="0" customHeight="1">
@@ -5853,16 +6397,16 @@
       </x:c>
     </x:row>
     <x:row r="28" ht="22.5" hidden="0" customHeight="1">
-      <x:c r="E28" s="914" t="str">
+      <x:c r="E28" s="1158" t="str">
         <x:v>Проверка</x:v>
       </x:c>
-      <x:c r="F28" s="914" t="str">
+      <x:c r="F28" s="1158" t="str">
         <x:v>Ожидается</x:v>
       </x:c>
-      <x:c r="G28" s="914" t="str">
+      <x:c r="G28" s="1158" t="str">
         <x:v>Факт</x:v>
       </x:c>
-      <x:c r="H28" s="914" t="str">
+      <x:c r="H28" s="1158" t="str">
         <x:v>Статус</x:v>
       </x:c>
     </x:row>
@@ -5871,12 +6415,12 @@
         <x:v>Закрепившаяся стоимость</x:v>
       </x:c>
       <x:c r="F29" s="377" t="n">
-        <x:f>'Калькулятор'!L27/'Калькулятор'!B12</x:f>
-        <x:v>40.411217576077</x:v>
+        <x:f>B16*B10</x:f>
+        <x:v>54.843795281818785</x:v>
       </x:c>
       <x:c r="G29" s="243" t="n">
         <x:f>B14</x:f>
-        <x:v>40.411217576077</x:v>
+        <x:v>54.84379528181877</x:v>
       </x:c>
       <x:c r="H29" s="236" t="str">
         <x:f>IF(ABS(G29-F29)&lt;0.01,"НОРМА","ПРОВЕРИТЬ")</x:f>
@@ -5888,12 +6432,12 @@
         <x:v>Полная стоимость пяти пакетов</x:v>
       </x:c>
       <x:c r="F30" s="377" t="n">
-        <x:f>'Калькулятор'!D31/'Калькулятор'!B12</x:f>
-        <x:v>49.78196721906139</x:v>
+        <x:f>SUM(F5:F9)*B10</x:f>
+        <x:v>67.56124122586903</x:v>
       </x:c>
       <x:c r="G30" s="243" t="n">
         <x:f>B13</x:f>
-        <x:v>49.7819672190614</x:v>
+        <x:v>67.56124122586903</x:v>
       </x:c>
       <x:c r="H30" s="236" t="str">
         <x:f>IF(ABS(G30-F30)&lt;0.01,"НОРМА","ПРОВЕРИТЬ")</x:f>
@@ -5902,15 +6446,15 @@
     </x:row>
     <x:row r="31" ht="19.5" hidden="0" customHeight="1">
       <x:c r="E31" t="str">
-        <x:v>Пакет равен окладу × множитель</x:v>
+        <x:v>Пакет равен окладу × множитель × результат</x:v>
       </x:c>
       <x:c r="F31" s="378" t="n">
-        <x:f>B5*B6</x:f>
-        <x:v>3.5</x:v>
+        <x:f>B5*B6*B7</x:f>
+        <x:v>4.75</x:v>
       </x:c>
       <x:c r="G31" s="243" t="n">
-        <x:f>B7</x:f>
-        <x:v>3.5</x:v>
+        <x:f>B8</x:f>
+        <x:v>4.75</x:v>
       </x:c>
       <x:c r="H31" s="236" t="str">
         <x:f>IF(ABS(G31-F31)&lt;0.000001,"НОРМА","ПРОВЕРИТЬ")</x:f>
@@ -5965,7 +6509,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="A1" s="898" t="str">
+      <x:c r="A1" s="1142" t="str">
         <x:v>LTI — правила, которым соответствует калькулятор</x:v>
       </x:c>
       <x:c r="B1" s="56"/>
@@ -5977,11 +6521,11 @@
       <x:c r="H1" s="56"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="951" t="str">
+      <x:c r="A2" s="1196" t="str">
         <x:v>Единый канон для документа, пятилетней модели и примеров</x:v>
       </x:c>
-      <x:c r="B2" s="951"/>
-      <x:c r="C2" s="951"/>
+      <x:c r="B2" s="1196"/>
+      <x:c r="C2" s="1196"/>
       <x:c r="D2" s="59"/>
       <x:c r="E2" s="59"/>
       <x:c r="F2" s="59"/>
@@ -5990,13 +6534,13 @@
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="914" t="str">
+      <x:c r="A4" s="1158" t="str">
         <x:v>Правило</x:v>
       </x:c>
-      <x:c r="B4" s="914" t="str">
+      <x:c r="B4" s="1158" t="str">
         <x:v>Как считается</x:v>
       </x:c>
-      <x:c r="C4" s="914" t="str">
+      <x:c r="C4" s="1158" t="str">
         <x:v>Что важно</x:v>
       </x:c>
     </x:row>
@@ -6019,7 +6563,7 @@
         <x:v>МИН(100%; 60% результата компании + 40% личного результата)</x:v>
       </x:c>
       <x:c r="C6" s="76" t="str">
-        <x:v>Отрицательный результат ограничен нулём</x:v>
+        <x:v>В примере: 60% × 90% + 40% × 102,5% = 95%</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25.5" hidden="0" customHeight="1">
@@ -6060,7 +6604,7 @@
         <x:v>Каждый год заново</x:v>
       </x:c>
       <x:c r="B10" s="76" t="str">
-        <x:v>Новое поимённое решение Совета</x:v>
+        <x:v>Новое решение по единым критериям: влияние на стоимость, критическая ответственность, измеримость и ценность удержания</x:v>
       </x:c>
       <x:c r="C10" s="76" t="str">
         <x:v>Нет вечного права на новый пакет</x:v>
@@ -6100,31 +6644,31 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="907" t="str">
+      <x:c r="A14" s="1151" t="str">
         <x:v>Плановая структура общего резерва — 5% / 4% / 1%</x:v>
       </x:c>
-      <x:c r="B14" s="907"/>
-      <x:c r="C14" s="907"/>
+      <x:c r="B14" s="1151"/>
+      <x:c r="C14" s="1151"/>
     </x:row>
     <x:row r="15" ht="39" customHeight="1">
-      <x:c r="A15" s="959" t="str">
+      <x:c r="A15" s="1207" t="str">
         <x:v>Назначение</x:v>
       </x:c>
-      <x:c r="B15" s="959" t="str">
+      <x:c r="B15" s="1207" t="str">
         <x:v>5% текущая команда · 4% будущие сильные наймы · 1% резерв Совета</x:v>
       </x:c>
-      <x:c r="C15" s="959" t="str">
+      <x:c r="C15" s="1207" t="str">
         <x:v>Это один предел 10%; перераспределение возможно только внутри него</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="914" t="str">
+      <x:c r="A16" s="1158" t="str">
         <x:v>Сверка</x:v>
       </x:c>
-      <x:c r="B16" s="914" t="str">
+      <x:c r="B16" s="1158" t="str">
         <x:v>Предыдущая версия</x:v>
       </x:c>
-      <x:c r="C16" s="914" t="str">
+      <x:c r="C16" s="1158" t="str">
         <x:v>Текущая версия</x:v>
       </x:c>
     </x:row>
@@ -6141,13 +6685,13 @@
     </x:row>
     <x:row r="18" ht="25.5" hidden="0" customHeight="1">
       <x:c r="A18" s="76" t="str">
-        <x:v>Средний пакет</x:v>
+        <x:v>Целевой и заработанный пакет</x:v>
       </x:c>
       <x:c r="B18" s="76" t="str">
         <x:v>Лестница ролей</x:v>
       </x:c>
       <x:c r="C18" s="76" t="str">
-        <x:v>5 млн ₽ × 0,7 = 3,5 млн ₽</x:v>
+        <x:v>5 млн ₽ × 1,0 × 95% = 4,75 млн ₽</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="25.5" hidden="0" customHeight="1">
@@ -6158,7 +6702,7 @@
         <x:v>Разовый набор 10/5/3/2</x:v>
       </x:c>
       <x:c r="C19" s="76" t="str">
-        <x:v>15 участников ежегодно в течение пяти лет</x:v>
+        <x:v>8 → 12 → 12 → 12 → 15 участников; всего 59 решений</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="25.5" hidden="0" customHeight="1">
@@ -6197,11 +6741,11 @@
     <x:row r="23"/>
     <x:row r="24"/>
     <x:row r="25" ht="39" hidden="0" customHeight="1">
-      <x:c r="A25" s="960" t="str">
+      <x:c r="A25" s="1208" t="str">
         <x:v>Последние пакеты к продаже закрепились не полностью: год 3 — 2/3, год 4 — 1/3, год 5 — 0. Модель не предполагает автоматического ускорения закрепления права.</x:v>
       </x:c>
-      <x:c r="B25" s="960"/>
-      <x:c r="C25" s="960"/>
+      <x:c r="B25" s="1208"/>
+      <x:c r="C25" s="1208"/>
       <x:c r="D25" s="75"/>
       <x:c r="E25" s="75"/>
       <x:c r="F25" s="75"/>
@@ -6234,7 +6778,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="A1" s="898" t="str">
+      <x:c r="A1" s="1142" t="str">
         <x:v>Ежегодные циклы LTI: пять решений Совета и контроль резерва</x:v>
       </x:c>
       <x:c r="B1" s="109"/>
@@ -6248,115 +6792,115 @@
       <x:c r="J1" s="109"/>
     </x:row>
     <x:row r="2" ht="27" hidden="0" customHeight="1">
-      <x:c r="A2" s="951" t="str">
+      <x:c r="A2" s="1196" t="str">
         <x:v>Каждый год — отдельное решение. Цена фиксируется на старте цикла, результат подтверждается после года, затем начинается 36-месячное закрепление права.</x:v>
       </x:c>
-      <x:c r="B2" s="951"/>
-      <x:c r="C2" s="951"/>
-      <x:c r="D2" s="951"/>
-      <x:c r="E2" s="951"/>
-      <x:c r="F2" s="951"/>
-      <x:c r="G2" s="951"/>
-      <x:c r="H2" s="951"/>
-      <x:c r="I2" s="951"/>
-      <x:c r="J2" s="951"/>
+      <x:c r="B2" s="1196"/>
+      <x:c r="C2" s="1196"/>
+      <x:c r="D2" s="1196"/>
+      <x:c r="E2" s="1196"/>
+      <x:c r="F2" s="1196"/>
+      <x:c r="G2" s="1196"/>
+      <x:c r="H2" s="1196"/>
+      <x:c r="I2" s="1196"/>
+      <x:c r="J2" s="1196"/>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="33" hidden="0" customHeight="1">
-      <x:c r="A4" s="961" t="str">
+      <x:c r="A4" s="1209" t="str">
         <x:v>Резерв LTI, млн расчётных ед.</x:v>
       </x:c>
-      <x:c r="B4" s="962" t="n">
+      <x:c r="B4" s="1210" t="n">
         <x:f>'Калькулятор'!B11</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C4" s="963" t="str">
+      <x:c r="C4" s="1211" t="str">
         <x:v>Занято к концу 5-го года</x:v>
       </x:c>
-      <x:c r="D4" s="962" t="n">
+      <x:c r="D4" s="1210" t="n">
         <x:f>'Калькулятор'!G27</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="E4" s="963" t="str">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="E4" s="1211" t="str">
         <x:v>Свободный резерв</x:v>
       </x:c>
-      <x:c r="F4" s="962" t="n">
+      <x:c r="F4" s="1210" t="n">
         <x:f>'Калькулятор'!I27</x:f>
-        <x:v>0.405515339487204</x:v>
-      </x:c>
-      <x:c r="G4" s="961" t="str">
+        <x:v>0.49545694889541103</x:v>
+      </x:c>
+      <x:c r="G4" s="1209" t="str">
         <x:v>Пиковое использование</x:v>
       </x:c>
-      <x:c r="H4" s="964" t="n">
+      <x:c r="H4" s="1212" t="n">
         <x:f>'Калькулятор'!H27</x:f>
-        <x:v>0.9594484660512796</x:v>
-      </x:c>
-      <x:c r="I4" s="961" t="str">
+        <x:v>0.9504543051104589</x:v>
+      </x:c>
+      <x:c r="I4" s="1209" t="str">
         <x:v>Статус</x:v>
       </x:c>
-      <x:c r="J4" s="965" t="str">
+      <x:c r="J4" s="1213" t="str">
         <x:f>'Калькулятор'!E42</x:f>
         <x:v>ПРОЙДЕНО</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="43.5" hidden="0" customHeight="1">
-      <x:c r="A5" s="960" t="str">
-        <x:v>Базовый сценарий занимает 9,594 из 10,000 млн расчётных единиц. 9,000 млн относятся к команде и найму; ещё 0,594 млн требуют отдельного решения Совета о переносе из его резерва. Остаётся 0,406 млн, или около 31,6 млн ₽ при продаже.</x:v>
-      </x:c>
-      <x:c r="B5" s="960"/>
-      <x:c r="C5" s="960"/>
-      <x:c r="D5" s="960"/>
-      <x:c r="E5" s="960"/>
-      <x:c r="F5" s="960"/>
-      <x:c r="G5" s="960"/>
-      <x:c r="H5" s="960"/>
-      <x:c r="I5" s="960"/>
-      <x:c r="J5" s="960"/>
+      <x:c r="A5" s="1208" t="str">
+        <x:v>Базовый сценарий занимает 9,505 из 10,000 млн расчётных единиц. 9,000 млн относятся к команде и найму; ещё 0,505 млн требуют отдельного решения Совета о переносе из его резерва. Остаётся 0,495 млн, или около 38,6 млн ₽ при продаже.</x:v>
+      </x:c>
+      <x:c r="B5" s="1208"/>
+      <x:c r="C5" s="1208"/>
+      <x:c r="D5" s="1208"/>
+      <x:c r="E5" s="1208"/>
+      <x:c r="F5" s="1208"/>
+      <x:c r="G5" s="1208"/>
+      <x:c r="H5" s="1208"/>
+      <x:c r="I5" s="1208"/>
+      <x:c r="J5" s="1208"/>
     </x:row>
     <x:row r="6"/>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="966" t="str">
-        <x:v>1. Ежегодное решение: 15 участников и средний пакет 0,7 оклада</x:v>
-      </x:c>
-      <x:c r="B7" s="1066"/>
-      <x:c r="C7" s="1066"/>
-      <x:c r="D7" s="1066"/>
-      <x:c r="E7" s="1066"/>
-      <x:c r="F7" s="1066"/>
-      <x:c r="G7" s="1066"/>
-      <x:c r="H7" s="1066"/>
-      <x:c r="I7" s="1066"/>
-      <x:c r="J7" s="1118"/>
+      <x:c r="A7" s="1214" t="str">
+        <x:v>1. Ежегодное решение: 8 → 12 → 12 → 12 → 15 участников и максимальный пакет 1,0 оклада</x:v>
+      </x:c>
+      <x:c r="B7" s="1325"/>
+      <x:c r="C7" s="1325"/>
+      <x:c r="D7" s="1325"/>
+      <x:c r="E7" s="1325"/>
+      <x:c r="F7" s="1325"/>
+      <x:c r="G7" s="1325"/>
+      <x:c r="H7" s="1325"/>
+      <x:c r="I7" s="1325"/>
+      <x:c r="J7" s="1326"/>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A8" s="914" t="str">
+      <x:c r="A8" s="1158" t="str">
         <x:v>Год</x:v>
       </x:c>
-      <x:c r="B8" s="914" t="str">
+      <x:c r="B8" s="1158" t="str">
         <x:v>Участников</x:v>
       </x:c>
-      <x:c r="C8" s="914" t="str">
+      <x:c r="C8" s="1158" t="str">
         <x:v>Оклад, млн ₽</x:v>
       </x:c>
-      <x:c r="D8" s="914" t="str">
+      <x:c r="D8" s="1158" t="str">
         <x:v>Множитель, ×</x:v>
       </x:c>
-      <x:c r="E8" s="914" t="str">
+      <x:c r="E8" s="1158" t="str">
         <x:v>Пакет на человека, млн ₽</x:v>
       </x:c>
-      <x:c r="F8" s="914" t="str">
+      <x:c r="F8" s="1158" t="str">
         <x:v>Пакеты на год, млн ₽</x:v>
       </x:c>
-      <x:c r="G8" s="914" t="str">
+      <x:c r="G8" s="1158" t="str">
         <x:v>Начальная цена, ₽</x:v>
       </x:c>
-      <x:c r="H8" s="914" t="str">
+      <x:c r="H8" s="1158" t="str">
         <x:v>Новые расчётные единицы, млн</x:v>
       </x:c>
-      <x:c r="I8" s="914" t="str">
+      <x:c r="I8" s="1158" t="str">
         <x:v>Занято накопительно, млн</x:v>
       </x:c>
-      <x:c r="J8" s="914" t="str">
+      <x:c r="J8" s="1158" t="str">
         <x:v>Использовано резерва</x:v>
       </x:c>
     </x:row>
@@ -6366,7 +6910,7 @@
       </x:c>
       <x:c r="B9" s="417" t="n">
         <x:f>'Калькулятор'!B22</x:f>
-        <x:v>15</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="399" t="n">
         <x:f>'Калькулятор'!B13</x:f>
@@ -6374,15 +6918,15 @@
       </x:c>
       <x:c r="D9" s="419" t="n">
         <x:f>'Калькулятор'!B14</x:f>
-        <x:v>0.7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="421" t="n">
         <x:f>C9*D9</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F9" s="422" t="n">
         <x:f>B9*E9</x:f>
-        <x:v>52.5</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G9" s="423" t="n">
         <x:f>'Калькулятор'!E22</x:f>
@@ -6390,15 +6934,15 @@
       </x:c>
       <x:c r="H9" s="421" t="n">
         <x:f>F9/G9</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="I9" s="421" t="n">
         <x:f>SUM($H$9:H9)</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="J9" s="280" t="n">
         <x:f>I9/'Калькулятор'!$B$11</x:f>
-        <x:v>0.4375</x:v>
+        <x:v>0.33333333333333337</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -6407,7 +6951,7 @@
       </x:c>
       <x:c r="B10" s="417" t="n">
         <x:f>'Калькулятор'!B23</x:f>
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C10" s="399" t="n">
         <x:f>'Калькулятор'!B13</x:f>
@@ -6415,15 +6959,15 @@
       </x:c>
       <x:c r="D10" s="419" t="n">
         <x:f>'Калькулятор'!B14</x:f>
-        <x:v>0.7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E10" s="421" t="n">
         <x:f>C10*D10</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F10" s="422" t="n">
         <x:f>B10*E10</x:f>
-        <x:v>52.5</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="G10" s="423" t="n">
         <x:f>'Калькулятор'!E23</x:f>
@@ -6431,15 +6975,15 @@
       </x:c>
       <x:c r="H10" s="421" t="n">
         <x:f>F10/G10</x:f>
-        <x:v>2.1875</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="I10" s="421" t="n">
         <x:f>SUM($H$9:H10)</x:f>
-        <x:v>6.5625</x:v>
+        <x:v>5.833333333333334</x:v>
       </x:c>
       <x:c r="J10" s="280" t="n">
         <x:f>I10/'Калькулятор'!$B$11</x:f>
-        <x:v>0.65625</x:v>
+        <x:v>0.5833333333333334</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -6448,7 +6992,7 @@
       </x:c>
       <x:c r="B11" s="417" t="n">
         <x:f>'Калькулятор'!B24</x:f>
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C11" s="399" t="n">
         <x:f>'Калькулятор'!B13</x:f>
@@ -6456,15 +7000,15 @@
       </x:c>
       <x:c r="D11" s="419" t="n">
         <x:f>'Калькулятор'!B14</x:f>
-        <x:v>0.7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E11" s="421" t="n">
         <x:f>C11*D11</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F11" s="422" t="n">
         <x:f>B11*E11</x:f>
-        <x:v>52.5</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="G11" s="423" t="n">
         <x:f>'Калькулятор'!E24</x:f>
@@ -6472,15 +7016,15 @@
       </x:c>
       <x:c r="H11" s="421" t="n">
         <x:f>F11/G11</x:f>
-        <x:v>1.3671875</x:v>
+        <x:v>1.5625</x:v>
       </x:c>
       <x:c r="I11" s="421" t="n">
         <x:f>SUM($H$9:H11)</x:f>
-        <x:v>7.9296875</x:v>
+        <x:v>7.395833333333334</x:v>
       </x:c>
       <x:c r="J11" s="280" t="n">
         <x:f>I11/'Калькулятор'!$B$11</x:f>
-        <x:v>0.79296875</x:v>
+        <x:v>0.7395833333333334</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -6489,7 +7033,7 @@
       </x:c>
       <x:c r="B12" s="417" t="n">
         <x:f>'Калькулятор'!B25</x:f>
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C12" s="399" t="n">
         <x:f>'Калькулятор'!B13</x:f>
@@ -6497,15 +7041,15 @@
       </x:c>
       <x:c r="D12" s="419" t="n">
         <x:f>'Калькулятор'!B14</x:f>
-        <x:v>0.7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E12" s="421" t="n">
         <x:f>C12*D12</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F12" s="422" t="n">
         <x:f>B12*E12</x:f>
-        <x:v>52.5</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="G12" s="423" t="n">
         <x:f>'Калькулятор'!E25</x:f>
@@ -6513,15 +7057,15 @@
       </x:c>
       <x:c r="H12" s="421" t="n">
         <x:f>F12/G12</x:f>
-        <x:v>0.9435017903645834</x:v>
+        <x:v>1.0782877604166667</x:v>
       </x:c>
       <x:c r="I12" s="421" t="n">
         <x:f>SUM($H$9:H12)</x:f>
-        <x:v>8.873189290364584</x:v>
+        <x:v>8.47412109375</x:v>
       </x:c>
       <x:c r="J12" s="280" t="n">
         <x:f>I12/'Калькулятор'!$B$11</x:f>
-        <x:v>0.8873189290364584</x:v>
+        <x:v>0.847412109375</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -6538,15 +7082,15 @@
       </x:c>
       <x:c r="D13" s="419" t="n">
         <x:f>'Калькулятор'!B14</x:f>
-        <x:v>0.7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E13" s="421" t="n">
         <x:f>C13*D13</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F13" s="422" t="n">
         <x:f>B13*E13</x:f>
-        <x:v>52.5</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="G13" s="423" t="n">
         <x:f>'Калькулятор'!E26</x:f>
@@ -6554,99 +7098,99 @@
       </x:c>
       <x:c r="H13" s="421" t="n">
         <x:f>F13/G13</x:f>
-        <x:v>0.7212953701482118</x:v>
+        <x:v>1.0304219573545883</x:v>
       </x:c>
       <x:c r="I13" s="421" t="n">
         <x:f>SUM($H$9:H13)</x:f>
-        <x:v>9.594484660512796</x:v>
+        <x:v>9.504543051104589</x:v>
       </x:c>
       <x:c r="J13" s="280" t="n">
         <x:f>I13/'Калькулятор'!$B$11</x:f>
-        <x:v>0.9594484660512796</x:v>
+        <x:v>0.9504543051104589</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="967" t="str">
+      <x:c r="A14" s="1215" t="str">
         <x:v>ИТОГО / СРЕДНЕЕ</x:v>
       </x:c>
-      <x:c r="B14" s="968" t="n">
+      <x:c r="B14" s="1216" t="n">
         <x:f>SUM(B9:B13)</x:f>
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="C14" s="969" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C14" s="1217" t="n">
         <x:f>AVERAGE(C9:C13)</x:f>
         <x:v>5</x:v>
       </x:c>
-      <x:c r="D14" s="970" t="n">
+      <x:c r="D14" s="1218" t="n">
         <x:f>AVERAGE(D9:D13)</x:f>
-        <x:v>0.7</x:v>
-      </x:c>
-      <x:c r="E14" s="972" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="1220" t="n">
         <x:f>AVERAGE(E9:E13)</x:f>
-        <x:v>3.5</x:v>
-      </x:c>
-      <x:c r="F14" s="972" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F14" s="1220" t="n">
         <x:f>SUM(F9:F13)</x:f>
-        <x:v>262.5</x:v>
-      </x:c>
-      <x:c r="G14" s="972"/>
-      <x:c r="H14" s="972" t="n">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="G14" s="1220"/>
+      <x:c r="H14" s="1220" t="n">
         <x:f>SUM(H9:H13)</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="I14" s="972" t="n">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="I14" s="1220" t="n">
         <x:f>MAX(I9:I13)</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="J14" s="933" t="n">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="J14" s="1178" t="n">
         <x:f>MAX(J9:J13)</x:f>
-        <x:v>0.9594484660512796</x:v>
+        <x:v>0.9504543051104589</x:v>
       </x:c>
     </x:row>
     <x:row r="15"/>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="966" t="str">
+      <x:c r="A16" s="1214" t="str">
         <x:v>2. Что закрепилось к продаже после пятого года</x:v>
       </x:c>
-      <x:c r="B16" s="1066"/>
-      <x:c r="C16" s="1066"/>
-      <x:c r="D16" s="1066"/>
-      <x:c r="E16" s="1066"/>
-      <x:c r="F16" s="1066"/>
-      <x:c r="G16" s="1066"/>
-      <x:c r="H16" s="1066"/>
-      <x:c r="I16" s="1066"/>
-      <x:c r="J16" s="1066"/>
+      <x:c r="B16" s="1325"/>
+      <x:c r="C16" s="1325"/>
+      <x:c r="D16" s="1325"/>
+      <x:c r="E16" s="1325"/>
+      <x:c r="F16" s="1325"/>
+      <x:c r="G16" s="1325"/>
+      <x:c r="H16" s="1325"/>
+      <x:c r="I16" s="1325"/>
+      <x:c r="J16" s="1325"/>
     </x:row>
     <x:row r="17" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A17" s="914" t="str">
+      <x:c r="A17" s="1158" t="str">
         <x:v>Год</x:v>
       </x:c>
-      <x:c r="B17" s="914" t="str">
+      <x:c r="B17" s="1158" t="str">
         <x:v>Выдано расчётных единиц, млн</x:v>
       </x:c>
-      <x:c r="C17" s="914" t="str">
+      <x:c r="C17" s="1158" t="str">
         <x:v>Закрепилось</x:v>
       </x:c>
-      <x:c r="D17" s="914" t="str">
+      <x:c r="D17" s="1158" t="str">
         <x:v>Закрепившиеся расчётные единицы, млн</x:v>
       </x:c>
-      <x:c r="E17" s="914" t="str">
+      <x:c r="E17" s="1158" t="str">
         <x:v>Незакрепившиеся расчётные единицы, млн</x:v>
       </x:c>
-      <x:c r="F17" s="914" t="str">
+      <x:c r="F17" s="1158" t="str">
         <x:v>Цена при продаже, ₽</x:v>
       </x:c>
-      <x:c r="G17" s="914" t="str">
+      <x:c r="G17" s="1158" t="str">
         <x:v>Закрепившаяся стоимость, млн ₽</x:v>
       </x:c>
-      <x:c r="H17" s="914" t="str">
+      <x:c r="H17" s="1158" t="str">
         <x:v>Незакрепившаяся стоимость, млн ₽</x:v>
       </x:c>
-      <x:c r="I17" s="914" t="str">
+      <x:c r="I17" s="1158" t="str">
         <x:v>Пояснение</x:v>
       </x:c>
-      <x:c r="J17" s="914" t="str">
+      <x:c r="J17" s="1158" t="str">
         <x:v>Статус</x:v>
       </x:c>
     </x:row>
@@ -6656,7 +7200,7 @@
       </x:c>
       <x:c r="B18" s="433" t="n">
         <x:f>'Калькулятор'!F22</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="C18" s="434" t="n">
         <x:f>'Калькулятор'!J22</x:f>
@@ -6664,7 +7208,7 @@
       </x:c>
       <x:c r="D18" s="421" t="n">
         <x:f>B18*C18</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="E18" s="421" t="n">
         <x:f>B18-D18</x:f>
@@ -6676,7 +7220,7 @@
       </x:c>
       <x:c r="G18" s="421" t="n">
         <x:f>D18*F18</x:f>
-        <x:v>340.50203990594486</x:v>
+        <x:v>259.43012564262466</x:v>
       </x:c>
       <x:c r="H18" s="421" t="n">
         <x:f>E18*F18</x:f>
@@ -6696,7 +7240,7 @@
       </x:c>
       <x:c r="B19" s="433" t="n">
         <x:f>'Калькулятор'!F23</x:f>
-        <x:v>2.1875</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="C19" s="434" t="n">
         <x:f>'Калькулятор'!J23</x:f>
@@ -6704,7 +7248,7 @@
       </x:c>
       <x:c r="D19" s="421" t="n">
         <x:f>B19*C19</x:f>
-        <x:v>2.1875</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="E19" s="421" t="n">
         <x:f>B19-D19</x:f>
@@ -6716,7 +7260,7 @@
       </x:c>
       <x:c r="G19" s="421" t="n">
         <x:f>D19*F19</x:f>
-        <x:v>170.25101995297243</x:v>
+        <x:v>194.57259423196848</x:v>
       </x:c>
       <x:c r="H19" s="421" t="n">
         <x:f>E19*F19</x:f>
@@ -6736,7 +7280,7 @@
       </x:c>
       <x:c r="B20" s="433" t="n">
         <x:f>'Калькулятор'!F24</x:f>
-        <x:v>1.3671875</x:v>
+        <x:v>1.5625</x:v>
       </x:c>
       <x:c r="C20" s="434" t="n">
         <x:f>'Калькулятор'!J24</x:f>
@@ -6744,11 +7288,11 @@
       </x:c>
       <x:c r="D20" s="421" t="n">
         <x:f>B20*C20</x:f>
-        <x:v>0.9114583333333333</x:v>
+        <x:v>1.0416666666666665</x:v>
       </x:c>
       <x:c r="E20" s="421" t="n">
         <x:f>B20-D20</x:f>
-        <x:v>0.45572916666666674</x:v>
+        <x:v>0.5208333333333335</x:v>
       </x:c>
       <x:c r="F20" s="423" t="n">
         <x:f>'Калькулятор'!$B$19/'Калькулятор'!$K$14</x:f>
@@ -6756,11 +7300,11 @@
       </x:c>
       <x:c r="G20" s="421" t="n">
         <x:f>D20*F20</x:f>
-        <x:v>70.93792498040517</x:v>
+        <x:v>81.0719142633202</x:v>
       </x:c>
       <x:c r="H20" s="421" t="n">
         <x:f>E20*F20</x:f>
-        <x:v>35.46896249020259</x:v>
+        <x:v>40.53595713166011</x:v>
       </x:c>
       <x:c r="I20" s="506" t="str">
         <x:v>Прошло 24 месяца</x:v>
@@ -6776,7 +7320,7 @@
       </x:c>
       <x:c r="B21" s="433" t="n">
         <x:f>'Калькулятор'!F25</x:f>
-        <x:v>0.9435017903645834</x:v>
+        <x:v>1.0782877604166667</x:v>
       </x:c>
       <x:c r="C21" s="434" t="n">
         <x:f>'Калькулятор'!J25</x:f>
@@ -6784,11 +7328,11 @@
       </x:c>
       <x:c r="D21" s="421" t="n">
         <x:f>B21*C21</x:f>
-        <x:v>0.3145005967881944</x:v>
+        <x:v>0.3594292534722222</x:v>
       </x:c>
       <x:c r="E21" s="421" t="n">
         <x:f>B21-D21</x:f>
-        <x:v>0.629001193576389</x:v>
+        <x:v>0.7188585069444445</x:v>
       </x:c>
       <x:c r="F21" s="423" t="n">
         <x:f>'Калькулятор'!$B$19/'Калькулятор'!$K$14</x:f>
@@ -6796,11 +7340,11 @@
       </x:c>
       <x:c r="G21" s="421" t="n">
         <x:f>D21*F21</x:f>
-        <x:v>24.477278801832515</x:v>
+        <x:v>27.97403291638002</x:v>
       </x:c>
       <x:c r="H21" s="421" t="n">
         <x:f>E21*F21</x:f>
-        <x:v>48.95455760366504</x:v>
+        <x:v>55.948065832760044</x:v>
       </x:c>
       <x:c r="I21" s="506" t="str">
         <x:v>Прошло 12 месяцев</x:v>
@@ -6816,7 +7360,7 @@
       </x:c>
       <x:c r="B22" s="433" t="n">
         <x:f>'Калькулятор'!F26</x:f>
-        <x:v>0.7212953701482118</x:v>
+        <x:v>1.0304219573545883</x:v>
       </x:c>
       <x:c r="C22" s="434" t="n">
         <x:f>'Калькулятор'!J26</x:f>
@@ -6828,7 +7372,7 @@
       </x:c>
       <x:c r="E22" s="421" t="n">
         <x:f>B22-D22</x:f>
-        <x:v>0.7212953701482118</x:v>
+        <x:v>1.0304219573545883</x:v>
       </x:c>
       <x:c r="F22" s="423" t="n">
         <x:f>'Калькулятор'!$B$19/'Калькулятор'!$K$14</x:f>
@@ -6840,7 +7384,7 @@
       </x:c>
       <x:c r="H22" s="421" t="n">
         <x:f>E22*F22</x:f>
-        <x:v>56.13772455089821</x:v>
+        <x:v>80.19674935842602</x:v>
       </x:c>
       <x:c r="I22" s="506" t="str">
         <x:v>Только подтверждение результата</x:v>
@@ -6851,76 +7395,76 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="28.5" hidden="0" customHeight="1">
-      <x:c r="A23" s="967" t="str">
+      <x:c r="A23" s="1215" t="str">
         <x:v>ИТОГО</x:v>
       </x:c>
-      <x:c r="B23" s="972" t="n">
+      <x:c r="B23" s="1220" t="n">
         <x:f>SUM(B18:B22)</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="C23" s="973"/>
-      <x:c r="D23" s="972" t="n">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="C23" s="1221"/>
+      <x:c r="D23" s="1220" t="n">
         <x:f>SUM(D18:D22)</x:f>
-        <x:v>7.788458930121528</x:v>
-      </x:c>
-      <x:c r="E23" s="972" t="n">
+        <x:v>7.234429253472222</x:v>
+      </x:c>
+      <x:c r="E23" s="1220" t="n">
         <x:f>SUM(E18:E22)</x:f>
-        <x:v>1.8060257303912675</x:v>
-      </x:c>
-      <x:c r="F23" s="972"/>
-      <x:c r="G23" s="972" t="n">
+        <x:v>2.2701137976323666</x:v>
+      </x:c>
+      <x:c r="F23" s="1220"/>
+      <x:c r="G23" s="1220" t="n">
         <x:f>SUM(G18:G22)</x:f>
-        <x:v>606.168263641155</x:v>
-      </x:c>
-      <x:c r="H23" s="972" t="n">
+        <x:v>563.0486670542933</x:v>
+      </x:c>
+      <x:c r="H23" s="1220" t="n">
         <x:f>SUM(H18:H22)</x:f>
-        <x:v>140.56124464476585</x:v>
-      </x:c>
-      <x:c r="I23" s="974" t="str">
+        <x:v>176.68077232284617</x:v>
+      </x:c>
+      <x:c r="I23" s="1222" t="str">
         <x:v>Последние пакеты закреплены не полностью</x:v>
       </x:c>
-      <x:c r="J23" s="975" t="str">
+      <x:c r="J23" s="1223" t="str">
         <x:v>ПРОВЕРЕНО</x:v>
       </x:c>
     </x:row>
     <x:row r="24"/>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="966" t="str">
+      <x:c r="A25" s="1214" t="str">
         <x:v>3. Источник цены: пять заданных раундов</x:v>
       </x:c>
-      <x:c r="B25" s="1066"/>
-      <x:c r="C25" s="1066"/>
-      <x:c r="D25" s="1066"/>
-      <x:c r="E25" s="1066"/>
-      <x:c r="F25" s="1118"/>
-      <x:c r="G25" s="1118"/>
-      <x:c r="H25" s="1118"/>
-      <x:c r="I25" s="1118"/>
-      <x:c r="J25" s="1118"/>
+      <x:c r="B25" s="1325"/>
+      <x:c r="C25" s="1325"/>
+      <x:c r="D25" s="1325"/>
+      <x:c r="E25" s="1325"/>
+      <x:c r="F25" s="1326"/>
+      <x:c r="G25" s="1326"/>
+      <x:c r="H25" s="1326"/>
+      <x:c r="I25" s="1326"/>
+      <x:c r="J25" s="1326"/>
     </x:row>
     <x:row r="26" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A26" s="914" t="str">
+      <x:c r="A26" s="1158" t="str">
         <x:v>Год</x:v>
       </x:c>
-      <x:c r="B26" s="914" t="str">
+      <x:c r="B26" s="1158" t="str">
         <x:v>Оценка до раунда, млн ₽</x:v>
       </x:c>
-      <x:c r="C26" s="914" t="str">
+      <x:c r="C26" s="1158" t="str">
         <x:v>Привлечено, млн ₽</x:v>
       </x:c>
-      <x:c r="D26" s="914" t="str">
+      <x:c r="D26" s="1158" t="str">
         <x:v>Оценка после раунда, млн ₽</x:v>
       </x:c>
-      <x:c r="E26" s="914" t="str">
+      <x:c r="E26" s="1158" t="str">
         <x:v>Расчётных единиц после раунда, млн</x:v>
       </x:c>
-      <x:c r="F26" s="914" t="str">
+      <x:c r="F26" s="1158" t="str">
         <x:v>Накопленное размытие</x:v>
       </x:c>
-      <x:c r="G26" s="914" t="str">
+      <x:c r="G26" s="1158" t="str">
         <x:v>Начальная цена, ₽</x:v>
       </x:c>
-      <x:c r="H26" s="914" t="str">
+      <x:c r="H26" s="1158" t="str">
         <x:v>Источник</x:v>
       </x:c>
     </x:row>
@@ -7086,48 +7630,48 @@
     </x:row>
     <x:row r="32"/>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
-      <x:c r="A33" s="976" t="str">
+      <x:c r="A33" s="1224" t="str">
         <x:v>Легенда: синий шрифт на голубом фоне — ввод; зелёный — ссылка на другой лист; чёрный — формула. Все пять раундов и 4 млрд ₽ инвестиций моделируются явно.</x:v>
       </x:c>
-      <x:c r="B33" s="976"/>
-      <x:c r="C33" s="976"/>
-      <x:c r="D33" s="976"/>
-      <x:c r="E33" s="976"/>
-      <x:c r="F33" s="976"/>
-      <x:c r="G33" s="976"/>
-      <x:c r="H33" s="976"/>
-      <x:c r="I33" s="976"/>
-      <x:c r="J33" s="976"/>
+      <x:c r="B33" s="1224"/>
+      <x:c r="C33" s="1224"/>
+      <x:c r="D33" s="1224"/>
+      <x:c r="E33" s="1224"/>
+      <x:c r="F33" s="1224"/>
+      <x:c r="G33" s="1224"/>
+      <x:c r="H33" s="1224"/>
+      <x:c r="I33" s="1224"/>
+      <x:c r="J33" s="1224"/>
     </x:row>
     <x:row r="34"/>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
-      <x:c r="A35" s="966" t="str">
+      <x:c r="A35" s="1214" t="str">
         <x:v>4. Контрольные проверки</x:v>
       </x:c>
-      <x:c r="B35" s="1066"/>
-      <x:c r="C35" s="1066"/>
-      <x:c r="D35" s="1066"/>
-      <x:c r="E35" s="1066"/>
-      <x:c r="F35" s="1118"/>
-      <x:c r="G35" s="1118"/>
-      <x:c r="H35" s="1118"/>
-      <x:c r="I35" s="1118"/>
-      <x:c r="J35" s="1118"/>
+      <x:c r="B35" s="1325"/>
+      <x:c r="C35" s="1325"/>
+      <x:c r="D35" s="1325"/>
+      <x:c r="E35" s="1325"/>
+      <x:c r="F35" s="1326"/>
+      <x:c r="G35" s="1326"/>
+      <x:c r="H35" s="1326"/>
+      <x:c r="I35" s="1326"/>
+      <x:c r="J35" s="1326"/>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
-      <x:c r="A36" s="914" t="str">
+      <x:c r="A36" s="1158" t="str">
         <x:v>Проверка</x:v>
       </x:c>
-      <x:c r="B36" s="914" t="str">
+      <x:c r="B36" s="1158" t="str">
         <x:v>Факт</x:v>
       </x:c>
-      <x:c r="C36" s="914" t="str">
+      <x:c r="C36" s="1158" t="str">
         <x:v>Ожидание / предел</x:v>
       </x:c>
-      <x:c r="D36" s="914" t="str">
+      <x:c r="D36" s="1158" t="str">
         <x:v>Отклонение</x:v>
       </x:c>
-      <x:c r="E36" s="914" t="str">
+      <x:c r="E36" s="1158" t="str">
         <x:v>Статус</x:v>
       </x:c>
     </x:row>
@@ -7157,7 +7701,7 @@
       </x:c>
       <x:c r="B38" s="421" t="n">
         <x:f>$D$4</x:f>
-        <x:v>9.594484660512796</x:v>
+        <x:v>9.504543051104589</x:v>
       </x:c>
       <x:c r="C38" s="421" t="n">
         <x:f>$B$4</x:f>
@@ -7165,7 +7709,7 @@
       </x:c>
       <x:c r="D38" s="421" t="n">
         <x:f>B38-C38</x:f>
-        <x:v>-0.405515339487204</x:v>
+        <x:v>-0.49545694889541103</x:v>
       </x:c>
       <x:c r="E38" s="429" t="str">
         <x:f>IF(B38&lt;=C38,"НОРМА","СТОП")</x:f>
@@ -7178,14 +7722,14 @@
       </x:c>
       <x:c r="B39" s="421" t="n">
         <x:f>$F$4</x:f>
-        <x:v>0.405515339487204</x:v>
+        <x:v>0.49545694889541103</x:v>
       </x:c>
       <x:c r="C39" s="421" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D39" s="421" t="n">
         <x:f>B39-C39</x:f>
-        <x:v>0.405515339487204</x:v>
+        <x:v>0.49545694889541103</x:v>
       </x:c>
       <x:c r="E39" s="429" t="str">
         <x:f>IF(B39&gt;=C39,"НОРМА","СТОП")</x:f>
@@ -7214,18 +7758,18 @@
     </x:row>
     <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A41" s="140" t="str">
-        <x:v>Занято примерно 96% резерва</x:v>
+        <x:v>Занято примерно 95% резерва</x:v>
       </x:c>
       <x:c r="B41" s="405" t="n">
         <x:f>$H$4</x:f>
-        <x:v>0.9594484660512796</x:v>
+        <x:v>0.9504543051104589</x:v>
       </x:c>
       <x:c r="C41" s="405" t="n">
-        <x:v>0.96</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="D41" s="405" t="n">
         <x:f>B41-C41</x:f>
-        <x:v>-0.0005515339487203175</x:v>
+        <x:v>0.0004543051104589635</x:v>
       </x:c>
       <x:c r="E41" s="429" t="str">
         <x:f>IF(ABS(D41)&lt;=0.005,"НОРМА","ПРОВЕРИТЬ")</x:f>
@@ -7233,31 +7777,31 @@
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
-      <x:c r="A42" s="977" t="str">
+      <x:c r="A42" s="1225" t="str">
         <x:v>СТАТУС МОДЕЛИ</x:v>
       </x:c>
-      <x:c r="B42" s="977"/>
-      <x:c r="C42" s="977"/>
-      <x:c r="D42" s="977"/>
-      <x:c r="E42" s="977" t="str">
+      <x:c r="B42" s="1225"/>
+      <x:c r="C42" s="1225"/>
+      <x:c r="D42" s="1225"/>
+      <x:c r="E42" s="1225" t="str">
         <x:f>IF(COUNTIF(E37:E41,"&lt;&gt;НОРМА")=0,"ПРОЙДЕНО","ПРОВЕРИТЬ")</x:f>
         <x:v>ПРОЙДЕНО</x:v>
       </x:c>
     </x:row>
     <x:row r="43"/>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
-      <x:c r="A44" s="966" t="str">
+      <x:c r="A44" s="1214" t="str">
         <x:v>5. Как читать подробную модель</x:v>
       </x:c>
-      <x:c r="B44" s="1066"/>
-      <x:c r="C44" s="1066"/>
-      <x:c r="D44" s="1066"/>
-      <x:c r="E44" s="1066"/>
-      <x:c r="F44" s="1066"/>
-      <x:c r="G44" s="1066"/>
-      <x:c r="H44" s="1066"/>
-      <x:c r="I44" s="1066"/>
-      <x:c r="J44" s="1066"/>
+      <x:c r="B44" s="1325"/>
+      <x:c r="C44" s="1325"/>
+      <x:c r="D44" s="1325"/>
+      <x:c r="E44" s="1325"/>
+      <x:c r="F44" s="1325"/>
+      <x:c r="G44" s="1325"/>
+      <x:c r="H44" s="1325"/>
+      <x:c r="I44" s="1325"/>
+      <x:c r="J44" s="1325"/>
     </x:row>
     <x:row r="45" ht="21" hidden="0" customHeight="1">
       <x:c r="A45" s="143" t="str">
@@ -7412,7 +7956,7 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25.5" customHeight="1">
-      <x:c r="A1" s="979" t="str">
+      <x:c r="A1" s="1227" t="str">
         <x:v>LTI: резерв 10% и пятилетний базовый сценарий</x:v>
       </x:c>
       <x:c r="B1" s="170"/>
@@ -7424,16 +7968,16 @@
       <x:c r="H1" s="170"/>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
-      <x:c r="A2" s="980" t="str">
+      <x:c r="A2" s="1228" t="str">
         <x:v>Как исходные 10 млн расчётных единиц распределяются, используются и закрепляются к продаже после пятого года.</x:v>
       </x:c>
-      <x:c r="B2" s="980"/>
-      <x:c r="C2" s="980"/>
-      <x:c r="D2" s="980"/>
-      <x:c r="E2" s="980"/>
-      <x:c r="F2" s="980"/>
-      <x:c r="G2" s="980"/>
-      <x:c r="H2" s="980"/>
+      <x:c r="B2" s="1228"/>
+      <x:c r="C2" s="1228"/>
+      <x:c r="D2" s="1228"/>
+      <x:c r="E2" s="1228"/>
+      <x:c r="F2" s="1228"/>
+      <x:c r="G2" s="1228"/>
+      <x:c r="H2" s="1228"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="168"/>
@@ -7446,33 +7990,33 @@
       <x:c r="H3" s="168"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="981" t="str">
+      <x:c r="A4" s="1229" t="str">
         <x:v>1. Масштаб общего резерва</x:v>
       </x:c>
-      <x:c r="B4" s="981"/>
-      <x:c r="C4" s="981"/>
-      <x:c r="D4" s="981"/>
-      <x:c r="E4" s="981"/>
-      <x:c r="F4" s="981"/>
-      <x:c r="G4" s="981" t="str">
+      <x:c r="B4" s="1229"/>
+      <x:c r="C4" s="1229"/>
+      <x:c r="D4" s="1229"/>
+      <x:c r="E4" s="1229"/>
+      <x:c r="F4" s="1229"/>
+      <x:c r="G4" s="1229" t="str">
         <x:v>Размытие за пять раундов</x:v>
       </x:c>
-      <x:c r="H4" s="1120" t="n">
+      <x:c r="H4" s="1328" t="n">
         <x:f>'Калькулятор'!L14</x:f>
         <x:v>0.5135685144200788</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="33" customHeight="1">
-      <x:c r="A5" s="982" t="str">
+      <x:c r="A5" s="1230" t="str">
         <x:v>Момент</x:v>
       </x:c>
-      <x:c r="B5" s="982" t="str">
+      <x:c r="B5" s="1230" t="str">
         <x:v>Стоимость капитала, млн ₽</x:v>
       </x:c>
-      <x:c r="C5" s="982" t="str">
+      <x:c r="C5" s="1230" t="str">
         <x:v>Доля резерва</x:v>
       </x:c>
-      <x:c r="D5" s="982" t="str">
+      <x:c r="D5" s="1230" t="str">
         <x:v>Стоимость резерва, млн ₽</x:v>
       </x:c>
       <x:c r="E5" s="179" t="str">
@@ -7494,16 +8038,16 @@
         <x:f>'Калькулятор'!B11/'Калькулятор'!B10</x:f>
         <x:v>0.1</x:v>
       </x:c>
-      <x:c r="D6" s="984" t="n">
+      <x:c r="D6" s="1232" t="n">
         <x:f>B6*C6</x:f>
         <x:v>120</x:v>
       </x:c>
-      <x:c r="E6" s="985" t="str">
+      <x:c r="E6" s="1233" t="str">
         <x:v>10 млн расчётных единиц из исходных 100 млн = 10% до раунда</x:v>
       </x:c>
-      <x:c r="F6" s="985"/>
-      <x:c r="G6" s="985"/>
-      <x:c r="H6" s="985"/>
+      <x:c r="F6" s="1233"/>
+      <x:c r="G6" s="1233"/>
+      <x:c r="H6" s="1233"/>
     </x:row>
     <x:row r="7" ht="28.5" customHeight="1">
       <x:c r="A7" s="183" t="str">
@@ -7517,16 +8061,16 @@
         <x:f>'Калькулятор'!B11/'Калькулятор'!K10</x:f>
         <x:v>0.075</x:v>
       </x:c>
-      <x:c r="D7" s="984" t="n">
+      <x:c r="D7" s="1232" t="n">
         <x:f>B7*C7</x:f>
         <x:v>120</x:v>
       </x:c>
-      <x:c r="E7" s="985" t="str">
+      <x:c r="E7" s="1233" t="str">
         <x:v>После первого выпуска те же 10 млн расчётных единиц = 7,5% компании</x:v>
       </x:c>
-      <x:c r="F7" s="985"/>
-      <x:c r="G7" s="985"/>
-      <x:c r="H7" s="985"/>
+      <x:c r="F7" s="1233"/>
+      <x:c r="G7" s="1233"/>
+      <x:c r="H7" s="1233"/>
     </x:row>
     <x:row r="8" ht="28.5" customHeight="1">
       <x:c r="A8" s="183" t="str">
@@ -7540,16 +8084,16 @@
         <x:f>'Калькулятор'!B11/'Калькулятор'!K14</x:f>
         <x:v>0.04864314855799212</x:v>
       </x:c>
-      <x:c r="D8" s="984" t="n">
+      <x:c r="D8" s="1232" t="n">
         <x:f>B8*C8</x:f>
         <x:v>778.2903769278739</x:v>
       </x:c>
-      <x:c r="E8" s="985" t="str">
+      <x:c r="E8" s="1233" t="str">
         <x:v>После всех пяти раундов те же 10 млн расчётных единиц = около 4,86% компании</x:v>
       </x:c>
-      <x:c r="F8" s="985"/>
-      <x:c r="G8" s="985"/>
-      <x:c r="H8" s="985"/>
+      <x:c r="F8" s="1233"/>
+      <x:c r="G8" s="1233"/>
+      <x:c r="H8" s="1233"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="168"/>
@@ -7562,37 +8106,37 @@
       <x:c r="H9" s="168"/>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="981" t="str">
+      <x:c r="A10" s="1229" t="str">
         <x:v>2. Плановое назначение единого резерва 10%</x:v>
       </x:c>
-      <x:c r="B10" s="981"/>
-      <x:c r="C10" s="981"/>
-      <x:c r="D10" s="981"/>
-      <x:c r="E10" s="981"/>
-      <x:c r="F10" s="981"/>
-      <x:c r="G10" s="981"/>
-      <x:c r="H10" s="981"/>
+      <x:c r="B10" s="1229"/>
+      <x:c r="C10" s="1229"/>
+      <x:c r="D10" s="1229"/>
+      <x:c r="E10" s="1229"/>
+      <x:c r="F10" s="1229"/>
+      <x:c r="G10" s="1229"/>
+      <x:c r="H10" s="1229"/>
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
-      <x:c r="A11" s="982" t="str">
+      <x:c r="A11" s="1230" t="str">
         <x:v>Кому</x:v>
       </x:c>
-      <x:c r="B11" s="982" t="str">
+      <x:c r="B11" s="1230" t="str">
         <x:v>Доля до первого раунда</x:v>
       </x:c>
-      <x:c r="C11" s="982" t="str">
+      <x:c r="C11" s="1230" t="str">
         <x:v>Расчётных единиц, млн</x:v>
       </x:c>
-      <x:c r="D11" s="982" t="str">
+      <x:c r="D11" s="1230" t="str">
         <x:v>Стоимость при 1,2 млрд ₽, млн ₽</x:v>
       </x:c>
-      <x:c r="E11" s="982" t="str">
+      <x:c r="E11" s="1230" t="str">
         <x:v>Доля после пяти раундов</x:v>
       </x:c>
-      <x:c r="F11" s="982" t="str">
+      <x:c r="F11" s="1230" t="str">
         <x:v>Стоимость при 16 млрд ₽, млн ₽</x:v>
       </x:c>
-      <x:c r="G11" s="982" t="str">
+      <x:c r="G11" s="1230" t="str">
         <x:v>Управление</x:v>
       </x:c>
       <x:c r="H11" s="179"/>
@@ -7601,7 +8145,7 @@
       <x:c r="A12" s="189" t="str">
         <x:v>Текущая команда</x:v>
       </x:c>
-      <x:c r="B12" s="986" t="n">
+      <x:c r="B12" s="1234" t="n">
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="C12" s="459" t="n">
@@ -7629,7 +8173,7 @@
       <x:c r="A13" s="190" t="str">
         <x:v>Будущие сильные наймы</x:v>
       </x:c>
-      <x:c r="B13" s="986" t="n">
+      <x:c r="B13" s="1234" t="n">
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="C13" s="461" t="n">
@@ -7657,7 +8201,7 @@
       <x:c r="A14" s="191" t="str">
         <x:v>Резерв Совета</x:v>
       </x:c>
-      <x:c r="B14" s="986" t="n">
+      <x:c r="B14" s="1234" t="n">
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="C14" s="463" t="n">
@@ -7682,30 +8226,30 @@
       <x:c r="H14" s="191"/>
     </x:row>
     <x:row r="15" ht="28.5" customHeight="1">
-      <x:c r="A15" s="987" t="str">
+      <x:c r="A15" s="1235" t="str">
         <x:v>ИТОГО</x:v>
       </x:c>
-      <x:c r="B15" s="988" t="n">
+      <x:c r="B15" s="1236" t="n">
         <x:f>SUM(B12:B14)</x:f>
         <x:v>0.09999999999999999</x:v>
       </x:c>
-      <x:c r="C15" s="991" t="n">
+      <x:c r="C15" s="1239" t="n">
         <x:f>SUM(C12:C14)</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D15" s="991" t="n">
+      <x:c r="D15" s="1239" t="n">
         <x:f>SUM(D12:D14)</x:f>
         <x:v>120</x:v>
       </x:c>
-      <x:c r="E15" s="992" t="n">
+      <x:c r="E15" s="1240" t="n">
         <x:f>SUM(E12:E14)</x:f>
         <x:v>0.048643148557992115</x:v>
       </x:c>
-      <x:c r="F15" s="991" t="n">
+      <x:c r="F15" s="1239" t="n">
         <x:f>SUM(F12:F14)</x:f>
         <x:v>778.290376927874</x:v>
       </x:c>
-      <x:c r="G15" s="991" t="str">
+      <x:c r="G15" s="1239" t="str">
         <x:v>Перераспределение возможно только внутри 10%</x:v>
       </x:c>
       <x:c r="H15" s="193"/>
@@ -7721,34 +8265,34 @@
       <x:c r="H16" s="168"/>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="981" t="str">
+      <x:c r="A17" s="1229" t="str">
         <x:v>3. Сверка базового сценария с назначением 5% / 4% / 1%</x:v>
       </x:c>
-      <x:c r="B17" s="981"/>
-      <x:c r="C17" s="981"/>
-      <x:c r="D17" s="981"/>
-      <x:c r="E17" s="981"/>
-      <x:c r="F17" s="981"/>
-      <x:c r="G17" s="981"/>
-      <x:c r="H17" s="981"/>
+      <x:c r="B17" s="1229"/>
+      <x:c r="C17" s="1229"/>
+      <x:c r="D17" s="1229"/>
+      <x:c r="E17" s="1229"/>
+      <x:c r="F17" s="1229"/>
+      <x:c r="G17" s="1229"/>
+      <x:c r="H17" s="1229"/>
     </x:row>
     <x:row r="18" ht="33" customHeight="1">
-      <x:c r="A18" s="982" t="str">
+      <x:c r="A18" s="1230" t="str">
         <x:v>Показатель</x:v>
       </x:c>
-      <x:c r="B18" s="982" t="str">
+      <x:c r="B18" s="1230" t="str">
         <x:v>Расчётных единиц, млн</x:v>
       </x:c>
-      <x:c r="C18" s="982" t="str">
+      <x:c r="C18" s="1230" t="str">
         <x:v>При продаже, млн ₽</x:v>
       </x:c>
-      <x:c r="D18" s="982" t="str">
+      <x:c r="D18" s="1230" t="str">
         <x:v>Что это значит</x:v>
       </x:c>
-      <x:c r="E18" s="982"/>
-      <x:c r="F18" s="982"/>
-      <x:c r="G18" s="982"/>
-      <x:c r="H18" s="982"/>
+      <x:c r="E18" s="1230"/>
+      <x:c r="F18" s="1230"/>
+      <x:c r="G18" s="1230"/>
+      <x:c r="H18" s="1230"/>
     </x:row>
     <x:row r="19" ht="31.5" customHeight="1">
       <x:c r="A19" s="188" t="str">
@@ -7756,14 +8300,14 @@
       </x:c>
       <x:c r="B19" s="651" t="n">
         <x:f>'Калькулятор'!G27</x:f>
-        <x:v>9.594484660512796</x:v>
+        <x:v>9.504543051104589</x:v>
       </x:c>
       <x:c r="C19" s="459" t="n">
         <x:f>B19*('Калькулятор'!$B$19/'Калькулятор'!$K$14)</x:f>
-        <x:v>746.7295082859209</x:v>
+        <x:v>739.7294393771396</x:v>
       </x:c>
       <x:c r="D19" s="188" t="str">
-        <x:v>15 участников ежегодно × 5 циклов</x:v>
+        <x:v>8 → 12 → 12 → 12 → 15 участников; 59 решений</x:v>
       </x:c>
       <x:c r="E19" s="188"/>
       <x:c r="F19" s="489"/>
@@ -7791,110 +8335,110 @@
       <x:c r="H20" s="650"/>
     </x:row>
     <x:row r="21" ht="39" customHeight="1">
-      <x:c r="A21" s="993" t="str">
+      <x:c r="A21" s="1241" t="str">
         <x:v>Требуется перенести из резерва Совета</x:v>
       </x:c>
-      <x:c r="B21" s="997" t="n">
+      <x:c r="B21" s="1245" t="n">
         <x:f>MAX(0,B19-B20)</x:f>
-        <x:v>0.594484660512796</x:v>
-      </x:c>
-      <x:c r="C21" s="996" t="n">
+        <x:v>0.504543051104589</x:v>
+      </x:c>
+      <x:c r="C21" s="1244" t="n">
         <x:f>B21*('Калькулятор'!$B$19/'Калькулятор'!$K$14)</x:f>
-        <x:v>46.268169050834324</x:v>
-      </x:c>
-      <x:c r="D21" s="993" t="str">
-        <x:v>0,594 млн расчётных единиц — только по отдельному решению Совета</x:v>
-      </x:c>
-      <x:c r="E21" s="993"/>
-      <x:c r="F21" s="993"/>
-      <x:c r="G21" s="993"/>
-      <x:c r="H21" s="996"/>
+        <x:v>39.268100142053015</x:v>
+      </x:c>
+      <x:c r="D21" s="1241" t="str">
+        <x:v>Около 0,505 млн расчётных единиц — только по отдельному решению Совета</x:v>
+      </x:c>
+      <x:c r="E21" s="1241"/>
+      <x:c r="F21" s="1241"/>
+      <x:c r="G21" s="1241"/>
+      <x:c r="H21" s="1244"/>
     </x:row>
     <x:row r="22" ht="31.5" customHeight="1">
-      <x:c r="A22" s="987" t="str">
+      <x:c r="A22" s="1235" t="str">
         <x:v>Остаётся в резерве Совета</x:v>
       </x:c>
-      <x:c r="B22" s="999" t="n">
+      <x:c r="B22" s="1247" t="n">
         <x:f>MAX(0,C14-B21)</x:f>
-        <x:v>0.405515339487204</x:v>
-      </x:c>
-      <x:c r="C22" s="991" t="n">
+        <x:v>0.49545694889541103</x:v>
+      </x:c>
+      <x:c r="C22" s="1239" t="n">
         <x:f>B22*('Калькулятор'!$B$19/'Калькулятор'!$K$14)</x:f>
-        <x:v>31.560868641953075</x:v>
-      </x:c>
-      <x:c r="D22" s="987" t="str">
+        <x:v>38.56093755073438</x:v>
+      </x:c>
+      <x:c r="D22" s="1235" t="str">
         <x:v>Свободный остаток базового сценария</x:v>
       </x:c>
-      <x:c r="E22" s="987"/>
-      <x:c r="F22" s="987"/>
-      <x:c r="G22" s="987"/>
-      <x:c r="H22" s="991"/>
+      <x:c r="E22" s="1235"/>
+      <x:c r="F22" s="1235"/>
+      <x:c r="G22" s="1235"/>
+      <x:c r="H22" s="1239"/>
     </x:row>
     <x:row r="23" ht="31.5" customHeight="1">
-      <x:c r="A23" s="1000" t="str">
+      <x:c r="A23" s="1248" t="str">
         <x:v>СВЕРКА</x:v>
       </x:c>
-      <x:c r="B23" s="1003" t="n">
+      <x:c r="B23" s="1251" t="n">
         <x:f>SUM(B20:B22)</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C23" s="1004" t="n">
+      <x:c r="C23" s="1252" t="n">
         <x:f>SUM(C20:C22)</x:f>
         <x:v>778.290376927874</x:v>
       </x:c>
-      <x:c r="D23" s="1000" t="str">
-        <x:v>9,000 + 0,594 + 0,406 = 10,000 млн расчётных единиц</x:v>
-      </x:c>
-      <x:c r="E23" s="1000"/>
-      <x:c r="F23" s="1000"/>
-      <x:c r="G23" s="1000"/>
-      <x:c r="H23" s="1000"/>
+      <x:c r="D23" s="1248" t="str">
+        <x:v>9,000 + 0,505 + 0,495 = 10,000 млн расчётных единиц</x:v>
+      </x:c>
+      <x:c r="E23" s="1248"/>
+      <x:c r="F23" s="1248"/>
+      <x:c r="G23" s="1248"/>
+      <x:c r="H23" s="1248"/>
     </x:row>
     <x:row r="24" ht="28.5" customHeight="1">
-      <x:c r="A24" s="1005"/>
-      <x:c r="B24" s="1006"/>
-      <x:c r="C24" s="1006"/>
-      <x:c r="D24" s="1007"/>
-      <x:c r="E24" s="1007"/>
-      <x:c r="F24" s="1008"/>
-      <x:c r="G24" s="1008"/>
-      <x:c r="H24" s="1009"/>
+      <x:c r="A24" s="1253"/>
+      <x:c r="B24" s="1254"/>
+      <x:c r="C24" s="1254"/>
+      <x:c r="D24" s="1255"/>
+      <x:c r="E24" s="1255"/>
+      <x:c r="F24" s="1256"/>
+      <x:c r="G24" s="1256"/>
+      <x:c r="H24" s="1257"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="981" t="str">
+      <x:c r="A25" s="1229" t="str">
         <x:v>4. Пять ежегодных решений: использование резерва и закрепление прав</x:v>
       </x:c>
-      <x:c r="B25" s="981"/>
-      <x:c r="C25" s="981"/>
-      <x:c r="D25" s="981"/>
-      <x:c r="E25" s="981"/>
-      <x:c r="F25" s="981"/>
-      <x:c r="G25" s="981"/>
-      <x:c r="H25" s="981"/>
+      <x:c r="B25" s="1229"/>
+      <x:c r="C25" s="1229"/>
+      <x:c r="D25" s="1229"/>
+      <x:c r="E25" s="1229"/>
+      <x:c r="F25" s="1229"/>
+      <x:c r="G25" s="1229"/>
+      <x:c r="H25" s="1229"/>
     </x:row>
     <x:row r="26" ht="39" customHeight="1">
-      <x:c r="A26" s="1010" t="str">
+      <x:c r="A26" s="1258" t="str">
         <x:v>Год</x:v>
       </x:c>
-      <x:c r="B26" s="1010" t="str">
+      <x:c r="B26" s="1258" t="str">
         <x:v>Участников</x:v>
       </x:c>
-      <x:c r="C26" s="1010" t="str">
+      <x:c r="C26" s="1258" t="str">
         <x:v>Новые расчётные единицы, млн</x:v>
       </x:c>
-      <x:c r="D26" s="1010" t="str">
+      <x:c r="D26" s="1258" t="str">
         <x:v>Занято накопительно, млн</x:v>
       </x:c>
-      <x:c r="E26" s="1010" t="str">
+      <x:c r="E26" s="1258" t="str">
         <x:v>Закрепилось к продаже</x:v>
       </x:c>
-      <x:c r="F26" s="1010" t="str">
+      <x:c r="F26" s="1258" t="str">
         <x:v>Закрепившиеся расчётные единицы, млн</x:v>
       </x:c>
-      <x:c r="G26" s="1010" t="str">
+      <x:c r="G26" s="1258" t="str">
         <x:v>Закрепившаяся стоимость, млн ₽</x:v>
       </x:c>
-      <x:c r="H26" s="1011" t="str">
+      <x:c r="H26" s="1259" t="str">
         <x:v>Пояснение</x:v>
       </x:c>
     </x:row>
@@ -7904,15 +8448,15 @@
       </x:c>
       <x:c r="B27" s="681" t="n">
         <x:f>'Калькулятор'!B22</x:f>
-        <x:v>15</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C27" s="651" t="n">
         <x:f>'Калькулятор'!F22</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="D27" s="651" t="n">
         <x:f>'Калькулятор'!G22</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="E27" s="690" t="n">
         <x:f>'Калькулятор'!J22</x:f>
@@ -7920,11 +8464,11 @@
       </x:c>
       <x:c r="F27" s="651" t="n">
         <x:f>'Калькулятор'!K22</x:f>
-        <x:v>4.375</x:v>
+        <x:v>3.3333333333333335</x:v>
       </x:c>
       <x:c r="G27" s="651" t="n">
         <x:f>'Калькулятор'!L22</x:f>
-        <x:v>340.50203990594486</x:v>
+        <x:v>259.43012564262466</x:v>
       </x:c>
       <x:c r="H27" s="672" t="str">
         <x:v>Закрепилось полностью</x:v>
@@ -7936,15 +8480,15 @@
       </x:c>
       <x:c r="B28" s="682" t="n">
         <x:f>'Калькулятор'!B23</x:f>
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C28" s="686" t="n">
         <x:f>'Калькулятор'!F23</x:f>
-        <x:v>2.1875</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="D28" s="686" t="n">
         <x:f>'Калькулятор'!G23</x:f>
-        <x:v>6.5625</x:v>
+        <x:v>5.833333333333334</x:v>
       </x:c>
       <x:c r="E28" s="691" t="n">
         <x:f>'Калькулятор'!J23</x:f>
@@ -7952,188 +8496,188 @@
       </x:c>
       <x:c r="F28" s="686" t="n">
         <x:f>'Калькулятор'!K23</x:f>
-        <x:v>2.1875</x:v>
+        <x:v>2.5</x:v>
       </x:c>
       <x:c r="G28" s="686" t="n">
         <x:f>'Калькулятор'!L23</x:f>
-        <x:v>170.25101995297243</x:v>
+        <x:v>194.57259423196848</x:v>
       </x:c>
       <x:c r="H28" s="673" t="str">
         <x:v>Закрепилось полностью</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="28.5" customHeight="1">
-      <x:c r="A29" s="993" t="n">
+      <x:c r="A29" s="1241" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B29" s="1013" t="n">
+      <x:c r="B29" s="1261" t="n">
         <x:f>'Калькулятор'!B24</x:f>
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C29" s="1014" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C29" s="1262" t="n">
         <x:f>'Калькулятор'!F24</x:f>
-        <x:v>1.3671875</x:v>
-      </x:c>
-      <x:c r="D29" s="1014" t="n">
+        <x:v>1.5625</x:v>
+      </x:c>
+      <x:c r="D29" s="1262" t="n">
         <x:f>'Калькулятор'!G24</x:f>
-        <x:v>7.9296875</x:v>
-      </x:c>
-      <x:c r="E29" s="1015" t="n">
+        <x:v>7.395833333333334</x:v>
+      </x:c>
+      <x:c r="E29" s="1263" t="n">
         <x:f>'Калькулятор'!J24</x:f>
         <x:v>0.6666666666666666</x:v>
       </x:c>
-      <x:c r="F29" s="1014" t="n">
+      <x:c r="F29" s="1262" t="n">
         <x:f>'Калькулятор'!K24</x:f>
-        <x:v>0.9114583333333333</x:v>
-      </x:c>
-      <x:c r="G29" s="1014" t="n">
+        <x:v>1.0416666666666665</x:v>
+      </x:c>
+      <x:c r="G29" s="1262" t="n">
         <x:f>'Калькулятор'!L24</x:f>
-        <x:v>70.93792498040517</x:v>
-      </x:c>
-      <x:c r="H29" s="1016" t="str">
+        <x:v>81.0719142633202</x:v>
+      </x:c>
+      <x:c r="H29" s="1264" t="str">
         <x:v>Закрепилось на 2/3</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="28.5" customHeight="1">
-      <x:c r="A30" s="1017" t="n">
+      <x:c r="A30" s="1265" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B30" s="1018" t="n">
+      <x:c r="B30" s="1266" t="n">
         <x:f>'Калькулятор'!B25</x:f>
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C30" s="1019" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C30" s="1267" t="n">
         <x:f>'Калькулятор'!F25</x:f>
-        <x:v>0.9435017903645834</x:v>
-      </x:c>
-      <x:c r="D30" s="1019" t="n">
+        <x:v>1.0782877604166667</x:v>
+      </x:c>
+      <x:c r="D30" s="1267" t="n">
         <x:f>'Калькулятор'!G25</x:f>
-        <x:v>8.873189290364584</x:v>
-      </x:c>
-      <x:c r="E30" s="1020" t="n">
+        <x:v>8.47412109375</x:v>
+      </x:c>
+      <x:c r="E30" s="1268" t="n">
         <x:f>'Калькулятор'!J25</x:f>
         <x:v>0.3333333333333333</x:v>
       </x:c>
-      <x:c r="F30" s="1019" t="n">
+      <x:c r="F30" s="1267" t="n">
         <x:f>'Калькулятор'!K25</x:f>
-        <x:v>0.3145005967881944</x:v>
-      </x:c>
-      <x:c r="G30" s="1019" t="n">
+        <x:v>0.3594292534722222</x:v>
+      </x:c>
+      <x:c r="G30" s="1267" t="n">
         <x:f>'Калькулятор'!L25</x:f>
-        <x:v>24.477278801832515</x:v>
-      </x:c>
-      <x:c r="H30" s="1021" t="str">
+        <x:v>27.97403291638002</x:v>
+      </x:c>
+      <x:c r="H30" s="1269" t="str">
         <x:v>Закрепилось на 1/3</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="28.5" customHeight="1">
-      <x:c r="A31" s="939" t="n">
+      <x:c r="A31" s="1184" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B31" s="1022" t="n">
+      <x:c r="B31" s="1270" t="n">
         <x:f>'Калькулятор'!B26</x:f>
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C31" s="1023" t="n">
+      <x:c r="C31" s="1271" t="n">
         <x:f>'Калькулятор'!F26</x:f>
-        <x:v>0.7212953701482118</x:v>
-      </x:c>
-      <x:c r="D31" s="1023" t="n">
+        <x:v>1.0304219573545883</x:v>
+      </x:c>
+      <x:c r="D31" s="1271" t="n">
         <x:f>'Калькулятор'!G26</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="E31" s="1024" t="n">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="E31" s="1272" t="n">
         <x:f>'Калькулятор'!J26</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F31" s="1023" t="n">
+      <x:c r="F31" s="1271" t="n">
         <x:f>'Калькулятор'!K26</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G31" s="1023" t="n">
+      <x:c r="G31" s="1271" t="n">
         <x:f>'Калькулятор'!L26</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H31" s="1025" t="str">
+      <x:c r="H31" s="1273" t="str">
         <x:v>К продаже ещё не закрепилось</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="28.5" customHeight="1">
-      <x:c r="A32" s="926" t="str">
+      <x:c r="A32" s="1171" t="str">
         <x:v>ИТОГО</x:v>
       </x:c>
-      <x:c r="B32" s="931" t="n">
+      <x:c r="B32" s="1176" t="n">
         <x:f>SUM(B27:B31)</x:f>
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="C32" s="932" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C32" s="1177" t="n">
         <x:f>SUM(C27:C31)</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="D32" s="932" t="n">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="D32" s="1177" t="n">
         <x:f>MAX(D27:D31)</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="E32" s="926"/>
-      <x:c r="F32" s="932" t="n">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="E32" s="1171"/>
+      <x:c r="F32" s="1177" t="n">
         <x:f>SUM(F27:F31)</x:f>
-        <x:v>7.788458930121528</x:v>
-      </x:c>
-      <x:c r="G32" s="932" t="n">
+        <x:v>7.234429253472222</x:v>
+      </x:c>
+      <x:c r="G32" s="1177" t="n">
         <x:f>SUM(G27:G31)</x:f>
-        <x:v>606.168263641155</x:v>
-      </x:c>
-      <x:c r="H32" s="1012" t="str">
+        <x:v>563.0486670542933</x:v>
+      </x:c>
+      <x:c r="H32" s="1260" t="str">
         <x:v>Последние три пакета закрепились не полностью</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="43.5" customHeight="1">
-      <x:c r="A33" s="960" t="str">
+      <x:c r="A33" s="1208" t="str">
         <x:v>Важно: новый пакет не возникает автоматически. Каждый цикл утверждается заново; закрепление права начинается после подтверждения результата и занимает 36 месяцев.</x:v>
       </x:c>
-      <x:c r="B33" s="960"/>
-      <x:c r="C33" s="960"/>
-      <x:c r="D33" s="960"/>
-      <x:c r="E33" s="960"/>
-      <x:c r="F33" s="960"/>
-      <x:c r="G33" s="960"/>
-      <x:c r="H33" s="960"/>
+      <x:c r="B33" s="1208"/>
+      <x:c r="C33" s="1208"/>
+      <x:c r="D33" s="1208"/>
+      <x:c r="E33" s="1208"/>
+      <x:c r="F33" s="1208"/>
+      <x:c r="G33" s="1208"/>
+      <x:c r="H33" s="1208"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="907" t="str">
+      <x:c r="A35" s="1151" t="str">
         <x:v>5. Чувствительность: что произойдёт, если цена расчётной единицы не растёт</x:v>
       </x:c>
-      <x:c r="B35" s="1118"/>
-      <x:c r="C35" s="1118"/>
-      <x:c r="D35" s="1118"/>
-      <x:c r="E35" s="1118"/>
-      <x:c r="F35" s="1118"/>
-      <x:c r="G35" s="1118"/>
-      <x:c r="H35" s="1118"/>
+      <x:c r="B35" s="1326"/>
+      <x:c r="C35" s="1326"/>
+      <x:c r="D35" s="1326"/>
+      <x:c r="E35" s="1326"/>
+      <x:c r="F35" s="1326"/>
+      <x:c r="G35" s="1326"/>
+      <x:c r="H35" s="1326"/>
     </x:row>
     <x:row r="36" ht="36" customHeight="1">
-      <x:c r="A36" s="914" t="str">
+      <x:c r="A36" s="1158" t="str">
         <x:v>Допущение</x:v>
       </x:c>
-      <x:c r="B36" s="914" t="str">
+      <x:c r="B36" s="1158" t="str">
         <x:v>Значение</x:v>
       </x:c>
-      <x:c r="C36" s="914" t="str">
+      <x:c r="C36" s="1158" t="str">
         <x:v>Как читать</x:v>
       </x:c>
-      <x:c r="D36" s="914" t="str">
+      <x:c r="D36" s="1158" t="str">
         <x:v>Показатель</x:v>
       </x:c>
-      <x:c r="E36" s="914" t="str">
+      <x:c r="E36" s="1158" t="str">
         <x:v>Итог / предел</x:v>
       </x:c>
-      <x:c r="F36" s="914" t="str">
+      <x:c r="F36" s="1158" t="str">
         <x:v>Доп. показатель</x:v>
       </x:c>
-      <x:c r="G36" s="914" t="str">
+      <x:c r="G36" s="1158" t="str">
         <x:v>Вывод</x:v>
       </x:c>
-      <x:c r="H36" s="914"/>
+      <x:c r="H36" s="1158"/>
     </x:row>
     <x:row r="37" ht="36" customHeight="1">
       <x:c r="A37" s="76" t="str">
@@ -8147,45 +8691,45 @@
         <x:v>Равна цене первого года</x:v>
       </x:c>
       <x:c r="D37" s="76" t="str">
-        <x:v>Пакетов по плану</x:v>
+        <x:v>Решений по плану</x:v>
       </x:c>
       <x:c r="E37" s="888" t="n">
-        <x:f>$B$38*$B$39</x:f>
-        <x:v>75</x:v>
+        <x:f>$B$38</x:f>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="F37" s="888" t="n">
-        <x:f>$B$38</x:f>
-        <x:v>15</x:v>
+        <x:f>E37/$B$39</x:f>
+        <x:v>11.8</x:v>
       </x:c>
       <x:c r="G37" s="76" t="str">
-        <x:v>15 × 5 = 75 пакетов</x:v>
+        <x:v>8 + 12 + 12 + 12 + 15 = 59 решений</x:v>
       </x:c>
       <x:c r="H37" s="76"/>
     </x:row>
     <x:row r="38" ht="36" customHeight="1">
       <x:c r="A38" s="76" t="str">
-        <x:v>Участников ежегодно</x:v>
+        <x:v>Всего решений за пять лет</x:v>
       </x:c>
       <x:c r="B38" s="884" t="n">
-        <x:f>'Калькулятор'!B12</x:f>
-        <x:v>15</x:v>
+        <x:f>'Калькулятор'!B27</x:f>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C38" s="76" t="str">
-        <x:v>Как в базовом сценарии</x:v>
+        <x:v>8 → 12 → 12 → 12 → 15</x:v>
       </x:c>
       <x:c r="D38" s="76" t="str">
         <x:v>Требуется расчётных единиц, млн</x:v>
       </x:c>
       <x:c r="E38" s="889" t="n">
         <x:f>E37*$B$42/$B$37</x:f>
-        <x:v>21.875</x:v>
+        <x:v>24.583333333333332</x:v>
       </x:c>
       <x:c r="F38" s="889" t="n">
         <x:f>E38/$B$39</x:f>
-        <x:v>4.375</x:v>
+        <x:v>4.916666666666666</x:v>
       </x:c>
       <x:c r="G38" s="76" t="str">
-        <x:v>75 × 3,5 млн ₽ ÷ 12 ₽</x:v>
+        <x:v>59 × 5 млн ₽ ÷ 12 ₽</x:v>
       </x:c>
       <x:c r="H38" s="76"/>
     </x:row>
@@ -8200,18 +8744,18 @@
       <x:c r="C39" s="76" t="str">
         <x:v>Пять ежегодных решений</x:v>
       </x:c>
-      <x:c r="D39" s="960" t="str">
+      <x:c r="D39" s="1208" t="str">
         <x:v>Использовано резерва</x:v>
       </x:c>
-      <x:c r="E39" s="1035" t="n">
+      <x:c r="E39" s="1283" t="n">
         <x:f>E38/'Калькулятор'!$B$11</x:f>
-        <x:v>2.1875</x:v>
-      </x:c>
-      <x:c r="F39" s="960"/>
-      <x:c r="G39" s="960" t="str">
+        <x:v>2.458333333333333</x:v>
+      </x:c>
+      <x:c r="F39" s="1208"/>
+      <x:c r="G39" s="1208" t="str">
         <x:v>Без роста резерв превышен более чем вдвое</x:v>
       </x:c>
-      <x:c r="H39" s="960"/>
+      <x:c r="H39" s="1208"/>
     </x:row>
     <x:row r="40" ht="36" customHeight="1">
       <x:c r="A40" s="76" t="str">
@@ -8224,18 +8768,18 @@
       <x:c r="C40" s="76" t="str">
         <x:v>Как в базовом сценарии</x:v>
       </x:c>
-      <x:c r="D40" s="952" t="str">
+      <x:c r="D40" s="1200" t="str">
         <x:v>Базовый сценарий с ростом цены</x:v>
       </x:c>
-      <x:c r="E40" s="1037" t="n">
+      <x:c r="E40" s="1285" t="n">
         <x:f>'Калькулятор'!H27</x:f>
-        <x:v>0.9594484660512796</x:v>
-      </x:c>
-      <x:c r="F40" s="952"/>
-      <x:c r="G40" s="952" t="str">
-        <x:v>9,594 млн из 10 млн расчётных единиц</x:v>
-      </x:c>
-      <x:c r="H40" s="952"/>
+        <x:v>0.9504543051104589</x:v>
+      </x:c>
+      <x:c r="F40" s="1200"/>
+      <x:c r="G40" s="1200" t="str">
+        <x:v>9,505 млн из 10 млн расчётных единиц</x:v>
+      </x:c>
+      <x:c r="H40" s="1200"/>
     </x:row>
     <x:row r="41" ht="46.5" customHeight="1">
       <x:c r="A41" s="76" t="str">
@@ -8243,26 +8787,26 @@
       </x:c>
       <x:c r="B41" s="887" t="n">
         <x:f>'Калькулятор'!B14</x:f>
-        <x:v>0.7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C41" s="76" t="str">
         <x:v>Как в базовом сценарии</x:v>
       </x:c>
-      <x:c r="D41" s="956" t="str">
-        <x:v>Основной предел: множитель при 15 участниках ежегодно</x:v>
-      </x:c>
-      <x:c r="E41" s="1049" t="n">
-        <x:f>$B$44*$B$37/($B$38*$B$39*$B$40)</x:f>
-        <x:v>0.288</x:v>
-      </x:c>
-      <x:c r="F41" s="1050" t="n">
+      <x:c r="D41" s="1204" t="str">
+        <x:v>Основной предел: множитель при 59 решениях</x:v>
+      </x:c>
+      <x:c r="E41" s="1290" t="n">
+        <x:f>$B$44*$B$37/($B$38*$B$40)</x:f>
+        <x:v>0.36610169491525424</x:v>
+      </x:c>
+      <x:c r="F41" s="1291" t="n">
         <x:f>E41*$B$40</x:f>
-        <x:v>1.44</x:v>
-      </x:c>
-      <x:c r="G41" s="956" t="str">
+        <x:v>1.8305084745762712</x:v>
+      </x:c>
+      <x:c r="G41" s="1204" t="str">
         <x:v>Сохраняет 1 млн расчётных единиц резерва Совета</x:v>
       </x:c>
-      <x:c r="H41" s="956"/>
+      <x:c r="H41" s="1204"/>
     </x:row>
     <x:row r="42" ht="46.5" customHeight="1">
       <x:c r="A42" s="76" t="str">
@@ -8270,26 +8814,26 @@
       </x:c>
       <x:c r="B42" s="888" t="n">
         <x:f>B40*B41</x:f>
-        <x:v>3.5</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C42" s="76" t="str">
         <x:v>Оклад × множитель</x:v>
       </x:c>
-      <x:c r="D42" s="956" t="str">
-        <x:v>Основной предел: полных решений при множителе 0,7</x:v>
-      </x:c>
-      <x:c r="E42" s="1051" t="n">
+      <x:c r="D42" s="1204" t="str">
+        <x:v>Основной предел: полные пакеты 1,0 зарплаты</x:v>
+      </x:c>
+      <x:c r="E42" s="1292" t="n">
         <x:f>INT($B$44*$B$37/$B$42)</x:f>
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="F42" s="1042" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F42" s="1293" t="n">
         <x:f>E42/$B$39</x:f>
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G42" s="956" t="str">
-        <x:v>30 решений за пять лет = 6 ежегодно</x:v>
-      </x:c>
-      <x:c r="H42" s="956"/>
+        <x:v>4.2</x:v>
+      </x:c>
+      <x:c r="G42" s="1204" t="str">
+        <x:v>21 полный пакет за пять лет; в среднем 4,2 в год</x:v>
+      </x:c>
+      <x:c r="H42" s="1204"/>
     </x:row>
     <x:row r="43" ht="46.5" customHeight="1">
       <x:c r="A43" s="1136" t="str">
@@ -8302,21 +8846,21 @@
       <x:c r="C43" s="1136" t="str">
         <x:v>Сохраняется для отдельных решений</x:v>
       </x:c>
-      <x:c r="D43" s="1047" t="str">
-        <x:v>Абсолютный верхний предел: множитель при 15 участниках ежегодно</x:v>
-      </x:c>
-      <x:c r="E43" s="1052" t="n">
-        <x:f>'Калькулятор'!$B$11*$B$37/($B$38*$B$39*$B$40)</x:f>
-        <x:v>0.32</x:v>
-      </x:c>
-      <x:c r="F43" s="1053" t="n">
+      <x:c r="D43" s="1294" t="str">
+        <x:v>Абсолютный верхний предел: множитель при 59 решениях</x:v>
+      </x:c>
+      <x:c r="E43" s="1299" t="n">
+        <x:f>'Калькулятор'!$B$11*$B$37/($B$38*$B$40)</x:f>
+        <x:v>0.4067796610169492</x:v>
+      </x:c>
+      <x:c r="F43" s="1300" t="n">
         <x:f>E43*$B$40</x:f>
-        <x:v>1.6</x:v>
-      </x:c>
-      <x:c r="G43" s="1047" t="str">
+        <x:v>2.0338983050847457</x:v>
+      </x:c>
+      <x:c r="G43" s="1294" t="str">
         <x:v>Требует расходования всех 10 млн расчётных единиц</x:v>
       </x:c>
-      <x:c r="H43" s="1047"/>
+      <x:c r="H43" s="1294"/>
     </x:row>
     <x:row r="44" ht="46.5" customHeight="1">
       <x:c r="A44" s="76" t="str">
@@ -8329,79 +8873,79 @@
       <x:c r="C44" s="76" t="str">
         <x:v>5% текущей команде + 4% будущим наймам</x:v>
       </x:c>
-      <x:c r="D44" s="1047" t="str">
-        <x:v>Абсолютный верхний предел: полных решений при множителе 0,7</x:v>
-      </x:c>
-      <x:c r="E44" s="1137" t="n">
+      <x:c r="D44" s="1294" t="str">
+        <x:v>Абсолютный верхний предел: полные пакеты 1,0 зарплаты</x:v>
+      </x:c>
+      <x:c r="E44" s="1301" t="n">
         <x:f>INT('Калькулятор'!$B$11*$B$37/$B$42)</x:f>
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="F44" s="1138" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F44" s="1302" t="n">
         <x:f>('Калькулятор'!$B$11*$B$37/$B$42)/$B$39</x:f>
-        <x:v>6.857142857142857</x:v>
-      </x:c>
-      <x:c r="G44" s="1047" t="str">
-        <x:v>34 полных решения; 6,9 в год — только теоретическая ёмкость</x:v>
-      </x:c>
-      <x:c r="H44" s="1047"/>
+        <x:v>4.8</x:v>
+      </x:c>
+      <x:c r="G44" s="1294" t="str">
+        <x:v>24 полных пакета; 4,8 в год — только теоретическая ёмкость</x:v>
+      </x:c>
+      <x:c r="H44" s="1294"/>
     </x:row>
     <x:row r="45" ht="58.5" customHeight="1">
-      <x:c r="A45" s="1060" t="str">
-        <x:v>Вывод: основной предел сохраняет 1 млн расчётных единиц резерва Совета — 30 полных решений, или 6 в год, при среднем пакете 0,288 оклада (1,44 млн ₽). Абсолютный предел при расходовании всех 10 млн — 34 полных решения, 6,9 теоретически в год и 0,32 оклада.</x:v>
-      </x:c>
-      <x:c r="B45" s="960"/>
-      <x:c r="C45" s="960"/>
-      <x:c r="D45" s="960"/>
-      <x:c r="E45" s="960"/>
-      <x:c r="F45" s="960"/>
-      <x:c r="G45" s="960"/>
-      <x:c r="H45" s="960"/>
+      <x:c r="A45" s="1303" t="str">
+        <x:v>Вывод: без роста цены 59 решений с пакетом 1,0 зарплаты потребуют 24,583 млн расчётных единиц, или 245,8% резерва. При сохранении 1 млн единиц Совету поместятся 21 полный пакет, либо средний пакет нужно снизить до 0,366 зарплаты. При расходовании всего резерва — 24 полных пакета или 0,407 зарплаты.</x:v>
+      </x:c>
+      <x:c r="B45" s="1208"/>
+      <x:c r="C45" s="1208"/>
+      <x:c r="D45" s="1208"/>
+      <x:c r="E45" s="1208"/>
+      <x:c r="F45" s="1208"/>
+      <x:c r="G45" s="1208"/>
+      <x:c r="H45" s="1208"/>
     </x:row>
     <x:row r="46" ht="39" customHeight="1">
-      <x:c r="A46" s="1062"/>
-      <x:c r="B46" s="1063"/>
-      <x:c r="C46" s="1063"/>
-      <x:c r="D46" s="1063"/>
-      <x:c r="E46" s="1063"/>
-      <x:c r="F46" s="1063"/>
-      <x:c r="G46" s="1063"/>
-      <x:c r="H46" s="1064"/>
+      <x:c r="A46" s="1304"/>
+      <x:c r="B46" s="1305"/>
+      <x:c r="C46" s="1305"/>
+      <x:c r="D46" s="1305"/>
+      <x:c r="E46" s="1305"/>
+      <x:c r="F46" s="1305"/>
+      <x:c r="G46" s="1305"/>
+      <x:c r="H46" s="1306"/>
     </x:row>
     <x:row r="47" ht="40.5" customHeight="1">
-      <x:c r="A47" s="966" t="str">
+      <x:c r="A47" s="1214" t="str">
         <x:v>6. Альтернатива продаже: денежный поток от дивидендов с года 5</x:v>
       </x:c>
-      <x:c r="B47" s="1126"/>
-      <x:c r="C47" s="1066"/>
-      <x:c r="D47" s="1118"/>
-      <x:c r="E47" s="1127"/>
-      <x:c r="F47" s="1128"/>
-      <x:c r="G47" s="1129"/>
-      <x:c r="H47" s="1066"/>
+      <x:c r="B47" s="1329"/>
+      <x:c r="C47" s="1325"/>
+      <x:c r="D47" s="1326"/>
+      <x:c r="E47" s="1330"/>
+      <x:c r="F47" s="1331"/>
+      <x:c r="G47" s="1332"/>
+      <x:c r="H47" s="1325"/>
     </x:row>
     <x:row r="48" ht="43.5" customHeight="1">
-      <x:c r="A48" s="914" t="str">
+      <x:c r="A48" s="1158" t="str">
         <x:v>Допущение</x:v>
       </x:c>
-      <x:c r="B48" s="1075" t="str">
+      <x:c r="B48" s="1307" t="str">
         <x:v>Значение</x:v>
       </x:c>
-      <x:c r="C48" s="914" t="str">
+      <x:c r="C48" s="1158" t="str">
         <x:v>Комментарий</x:v>
       </x:c>
-      <x:c r="D48" s="914" t="str">
+      <x:c r="D48" s="1158" t="str">
         <x:v>Год</x:v>
       </x:c>
-      <x:c r="E48" s="1103" t="str">
+      <x:c r="E48" s="1314" t="str">
         <x:v>Закрепившиеся расчётные единицы, млн</x:v>
       </x:c>
-      <x:c r="F48" s="1104" t="str">
+      <x:c r="F48" s="1315" t="str">
         <x:v>Доля компании</x:v>
       </x:c>
-      <x:c r="G48" s="1075" t="str">
+      <x:c r="G48" s="1307" t="str">
         <x:v>Поток всей команде до личных налогов, млн ₽</x:v>
       </x:c>
-      <x:c r="H48" s="914" t="str">
+      <x:c r="H48" s="1158" t="str">
         <x:v>Поток одному постоянному участнику, млн ₽</x:v>
       </x:c>
     </x:row>
@@ -8409,7 +8953,7 @@
       <x:c r="A49" s="76" t="str">
         <x:v>Начало выплат, год</x:v>
       </x:c>
-      <x:c r="B49" s="1083" t="n">
+      <x:c r="B49" s="1308" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="C49" s="76" t="str">
@@ -8420,26 +8964,26 @@
       </x:c>
       <x:c r="E49" s="1140" t="n">
         <x:f>'Калькулятор'!K27</x:f>
-        <x:v>7.788458930121528</x:v>
+        <x:v>7.234429253472222</x:v>
       </x:c>
       <x:c r="F49" s="1141" t="n">
         <x:f>E49/('Калькулятор'!$K$14*(1+$B$52)^(D49-$B$49))</x:f>
-        <x:v>0.037885516477572184</x:v>
-      </x:c>
-      <x:c r="G49" s="1086" t="n">
+        <x:v>0.035190541690893334</x:v>
+      </x:c>
+      <x:c r="G49" s="1313" t="n">
         <x:f>$B$53*F49</x:f>
-        <x:v>37.88551647757218</x:v>
-      </x:c>
-      <x:c r="H49" s="1115" t="n">
-        <x:f>G49/'Калькулятор'!$B$12</x:f>
-        <x:v>2.525701098504812</x:v>
+        <x:v>35.19054169089333</x:v>
+      </x:c>
+      <x:c r="H49" s="1320" t="n">
+        <x:f>$B$53*('Один пакет'!F5+'Один пакет'!F6+'Один пакет'!F7*2/3+'Один пакет'!F8*1/3)/'Калькулятор'!$K$14</x:f>
+        <x:v>3.427737205113674</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="40.5" customHeight="1">
       <x:c r="A50" s="76" t="str">
         <x:v>Прибыль ежегодно, млн ₽</x:v>
       </x:c>
-      <x:c r="B50" s="1084" t="n">
+      <x:c r="B50" s="1309" t="n">
         <x:v>2000</x:v>
       </x:c>
       <x:c r="C50" s="76" t="str">
@@ -8450,26 +8994,26 @@
       </x:c>
       <x:c r="E50" s="1140" t="n">
         <x:f>'Калькулятор'!F22+'Калькулятор'!F23+'Калькулятор'!F24+'Калькулятор'!F25*2/3+'Калькулятор'!F26*1/3</x:f>
-        <x:v>8.799120483625794</x:v>
+        <x:v>8.458165826062642</x:v>
       </x:c>
       <x:c r="F50" s="1141" t="n">
         <x:f>E50/('Калькулятор'!$K$14*(1+$B$52)^(D50-$B$49))</x:f>
-        <x:v>0.0428016924864681</x:v>
-      </x:c>
-      <x:c r="G50" s="1086" t="n">
+        <x:v>0.041143181680529724</x:v>
+      </x:c>
+      <x:c r="G50" s="1313" t="n">
         <x:f>$B$53*F50</x:f>
-        <x:v>42.8016924864681</x:v>
-      </x:c>
-      <x:c r="H50" s="1115" t="n">
-        <x:f>G50/'Калькулятор'!$B$12</x:f>
-        <x:v>2.85344616576454</x:v>
+        <x:v>41.14318168052972</x:v>
+      </x:c>
+      <x:c r="H50" s="1320" t="n">
+        <x:f>$B$53*('Один пакет'!F5+'Один пакет'!F6+'Один пакет'!F7+'Один пакет'!F8*2/3+'Один пакет'!F9*1/3)/'Калькулятор'!$K$14</x:f>
+        <x:v>3.8725340821090173</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="40.5" customHeight="1">
       <x:c r="A51" s="1139" t="str">
         <x:v>Доля прибыли владельцам</x:v>
       </x:c>
-      <x:c r="B51" s="1085" t="n">
+      <x:c r="B51" s="1310" t="n">
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="C51" s="1139" t="str">
@@ -8480,26 +9024,26 @@
       </x:c>
       <x:c r="E51" s="1111" t="n">
         <x:f>SUM('Калькулятор'!F22:F25)+'Калькулятор'!F26*2/3</x:f>
-        <x:v>9.354052870463391</x:v>
+        <x:v>9.161069065319726</x:v>
       </x:c>
       <x:c r="F51" s="1113" t="n">
         <x:f>E51/('Калькулятор'!$K$14*(1+$B$52)^(D51-$B$49))</x:f>
-        <x:v>0.045501058339726334</x:v>
-      </x:c>
-      <x:c r="G51" s="1086" t="n">
+        <x:v>0.04456232434943735</x:v>
+      </x:c>
+      <x:c r="G51" s="1313" t="n">
         <x:f>$B$53*F51</x:f>
-        <x:v>45.501058339726335</x:v>
-      </x:c>
-      <x:c r="H51" s="1115" t="n">
-        <x:f>G51/'Калькулятор'!$B$12</x:f>
-        <x:v>3.033403889315089</x:v>
+        <x:v>44.56232434943735</x:v>
+      </x:c>
+      <x:c r="H51" s="1320" t="n">
+        <x:f>$B$53*(SUM('Один пакет'!F5:F8)+'Один пакет'!F9*2/3)/'Калькулятор'!$K$14</x:f>
+        <x:v>4.116762421213335</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="40.5" customHeight="1">
       <x:c r="A52" s="1139" t="str">
         <x:v>Рост числа расчётных единиц после года 5</x:v>
       </x:c>
-      <x:c r="B52" s="1085" t="n">
+      <x:c r="B52" s="1310" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C52" s="1139" t="str">
@@ -8510,95 +9054,95 @@
       </x:c>
       <x:c r="E52" s="1111" t="n">
         <x:f>SUM('Калькулятор'!F22:F26)</x:f>
-        <x:v>9.594484660512796</x:v>
+        <x:v>9.504543051104589</x:v>
       </x:c>
       <x:c r="F52" s="1113" t="n">
         <x:f>E52/('Калькулятор'!$K$14*(1+$B$52)^(D52-$B$49))</x:f>
-        <x:v>0.046670594267870055</x:v>
-      </x:c>
-      <x:c r="G52" s="1086" t="n">
+        <x:v>0.04623308996107122</x:v>
+      </x:c>
+      <x:c r="G52" s="1313" t="n">
         <x:f>$B$53*F52</x:f>
-        <x:v>46.67059426787006</x:v>
-      </x:c>
-      <x:c r="H52" s="1115" t="n">
-        <x:f>G52/'Калькулятор'!$B$12</x:f>
-        <x:v>3.111372951191337</x:v>
+        <x:v>46.23308996107122</x:v>
+      </x:c>
+      <x:c r="H52" s="1320" t="n">
+        <x:f>$B$53*SUM('Один пакет'!F5:F9)/'Калькулятор'!$K$14</x:f>
+        <x:v>4.222577576616813</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="40.5" customHeight="1">
-      <x:c r="A53" s="952" t="str">
+      <x:c r="A53" s="1200" t="str">
         <x:v>Общая сумма владельцам ежегодно, млн ₽</x:v>
       </x:c>
-      <x:c r="B53" s="1086" t="n">
+      <x:c r="B53" s="1313" t="n">
         <x:f>B50*B51</x:f>
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="C53" s="952" t="str">
+      <x:c r="C53" s="1200" t="str">
         <x:v>Прибыль × доля владельцам</x:v>
       </x:c>
-      <x:c r="D53" s="952" t="str">
+      <x:c r="D53" s="1200" t="str">
         <x:v>8 и далее</x:v>
       </x:c>
-      <x:c r="E53" s="1112" t="n">
+      <x:c r="E53" s="1323" t="n">
         <x:f>E52</x:f>
-        <x:v>9.594484660512796</x:v>
-      </x:c>
-      <x:c r="F53" s="1114" t="n">
+        <x:v>9.504543051104589</x:v>
+      </x:c>
+      <x:c r="F53" s="1324" t="n">
         <x:f>F52</x:f>
-        <x:v>0.046670594267870055</x:v>
-      </x:c>
-      <x:c r="G53" s="1086" t="n">
+        <x:v>0.04623308996107122</x:v>
+      </x:c>
+      <x:c r="G53" s="1313" t="n">
         <x:f>G52</x:f>
-        <x:v>46.67059426787006</x:v>
-      </x:c>
-      <x:c r="H53" s="1115" t="n">
+        <x:v>46.23308996107122</x:v>
+      </x:c>
+      <x:c r="H53" s="1320" t="n">
         <x:f>H52</x:f>
-        <x:v>3.111372951191337</x:v>
+        <x:v>4.222577576616813</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="43.5" customHeight="1">
-      <x:c r="A54" s="952" t="str">
-        <x:v>Личный пример: один постоянный участник получает один равный пакет каждый год и остаётся все пять лет.</x:v>
-      </x:c>
-      <x:c r="B54" s="952"/>
-      <x:c r="C54" s="952"/>
-      <x:c r="D54" s="952" t="str">
+      <x:c r="A54" s="1200" t="str">
+        <x:v>Личный пример: Мария ежегодно получает целевой пакет 1,0 зарплаты, зарабатывает 95% и остаётся все пять лет.</x:v>
+      </x:c>
+      <x:c r="B54" s="1200"/>
+      <x:c r="C54" s="1200"/>
+      <x:c r="D54" s="1200" t="str">
         <x:v>ИТОГО 5–8</x:v>
       </x:c>
-      <x:c r="E54" s="952"/>
-      <x:c r="F54" s="952"/>
-      <x:c r="G54" s="1086" t="n">
+      <x:c r="E54" s="1200"/>
+      <x:c r="F54" s="1200"/>
+      <x:c r="G54" s="1313" t="n">
         <x:f>SUM(G49:G52)</x:f>
-        <x:v>172.85886157163668</x:v>
-      </x:c>
-      <x:c r="H54" s="1115" t="n">
+        <x:v>167.1291376819316</x:v>
+      </x:c>
+      <x:c r="H54" s="1320" t="n">
         <x:f>SUM(H49:H52)</x:f>
-        <x:v>11.523924104775778</x:v>
+        <x:v>15.63961128505284</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="46.5" customHeight="1">
-      <x:c r="A55" s="952" t="str">
-        <x:v>При неизменной прибыли 2 млрд ₽, доле выплат 50% и отсутствии новых размытий поток всей команде с года 8 остаётся около 46,7 млн ₽ ежегодно, а одному постоянному участнику — около 3,11 млн ₽ ежегодно до личных налогов.</x:v>
-      </x:c>
-      <x:c r="B55" s="952"/>
-      <x:c r="C55" s="952"/>
-      <x:c r="D55" s="952"/>
-      <x:c r="E55" s="952"/>
-      <x:c r="F55" s="952"/>
-      <x:c r="G55" s="952"/>
-      <x:c r="H55" s="952"/>
+      <x:c r="A55" s="1200" t="str">
+        <x:v>При неизменной прибыли 2 млрд ₽, доле выплат 50% и отсутствии новых размытий поток всей команде с года 8 остаётся около 46,2 млн ₽ ежегодно, а Марии — около 4,22 млн ₽ ежегодно до личных налогов.</x:v>
+      </x:c>
+      <x:c r="B55" s="1200"/>
+      <x:c r="C55" s="1200"/>
+      <x:c r="D55" s="1200"/>
+      <x:c r="E55" s="1200"/>
+      <x:c r="F55" s="1200"/>
+      <x:c r="G55" s="1200"/>
+      <x:c r="H55" s="1200"/>
     </x:row>
     <x:row r="56" ht="82.5" customHeight="1">
-      <x:c r="A56" s="956" t="str">
-        <x:v>Дивиденды не гарантированы. Каждый год они зависят от фактической прибыли и денег, корпоративных решений, требований закона и прав инвесторов. Прибыль до процентов, налогов и амортизации не равна прибыли, доступной для распределения: 2 млрд ₽ — отдельное условное допущение дивидендного сценария, а не автоматическое следствие этого показателя. Личный пример предполагает один равный пакет ежегодно, непрерывное участие все пять лет и суммы до личных налогов.</x:v>
-      </x:c>
-      <x:c r="B56" s="956"/>
-      <x:c r="C56" s="956"/>
-      <x:c r="D56" s="956"/>
-      <x:c r="E56" s="956"/>
-      <x:c r="F56" s="956"/>
-      <x:c r="G56" s="956"/>
-      <x:c r="H56" s="956"/>
+      <x:c r="A56" s="1204" t="str">
+        <x:v>Дивиденды не гарантированы. Каждый год они зависят от фактической прибыли и денег, корпоративных решений, требований закона и прав инвесторов. Прибыль до процентов, налогов и амортизации не равна прибыли, доступной для распределения: 2 млрд ₽ — отдельное условное допущение дивидендного сценария, а не автоматическое следствие этого показателя. Личный пример предполагает пакет 4,75 млн ₽ ежегодно, непрерывное участие все пять лет и суммы до личных налогов.</x:v>
+      </x:c>
+      <x:c r="B56" s="1204"/>
+      <x:c r="C56" s="1204"/>
+      <x:c r="D56" s="1204"/>
+      <x:c r="E56" s="1204"/>
+      <x:c r="F56" s="1204"/>
+      <x:c r="G56" s="1204"/>
+      <x:c r="H56" s="1204"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>